<commit_message>
Use Yahoo-style period convention for weekly/monthly/yearly data
Date column is the first trading day of the period, values come from the
last trading day, and Combined aligns on Monday / 1st of month / Jan 1.

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/sample/PortfolioData_W_20260803_20260831_SAMPLE.xlsx
+++ b/sample/PortfolioData_W_20260803_20260831_SAMPLE.xlsx
@@ -546,7 +546,7 @@
         </is>
       </c>
       <c r="F2" s="2" t="n">
-        <v>46234</v>
+        <v>46230</v>
       </c>
       <c r="G2" s="2" t="n">
         <v>46265</v>
@@ -556,7 +556,7 @@
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>示範：2026-08-21 該週最後交易日為 08-20 / demo: last trading day of the week is 08-20</t>
+          <t>示範：2026-08-17 該週週一休市，日期欄標 08-18（第一個交易日），Combined 仍在 08-17 / demo: Monday closed, date is 08-18, Combined stays at 08-17</t>
         </is>
       </c>
     </row>
@@ -587,7 +587,7 @@
         </is>
       </c>
       <c r="F3" s="2" t="n">
-        <v>46234</v>
+        <v>46230</v>
       </c>
       <c r="G3" s="2" t="n">
         <v>46265</v>
@@ -597,7 +597,7 @@
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>示範：2026-08-14 該週整週休市，Combined 留白 / demo: whole week closed, blank in Combined</t>
+          <t>示範：2026-08-10 該週整週休市，Combined 留白 / demo: whole week closed, blank in Combined</t>
         </is>
       </c>
     </row>
@@ -628,7 +628,7 @@
         </is>
       </c>
       <c r="F4" s="2" t="n">
-        <v>46234</v>
+        <v>46230</v>
       </c>
       <c r="G4" s="2" t="n">
         <v>46265</v>
@@ -665,7 +665,7 @@
         </is>
       </c>
       <c r="F5" s="2" t="n">
-        <v>46234</v>
+        <v>46230</v>
       </c>
       <c r="G5" s="2" t="n">
         <v>46265</v>
@@ -702,7 +702,7 @@
         </is>
       </c>
       <c r="F6" s="2" t="n">
-        <v>46234</v>
+        <v>46230</v>
       </c>
       <c r="G6" s="2" t="n">
         <v>46265</v>
@@ -739,7 +739,7 @@
         </is>
       </c>
       <c r="F7" s="2" t="n">
-        <v>46234</v>
+        <v>46230</v>
       </c>
       <c r="G7" s="2" t="n">
         <v>46265</v>
@@ -776,7 +776,7 @@
         </is>
       </c>
       <c r="F8" s="2" t="n">
-        <v>46234</v>
+        <v>46230</v>
       </c>
       <c r="G8" s="2" t="n">
         <v>46265</v>
@@ -813,7 +813,7 @@
         </is>
       </c>
       <c r="F9" s="2" t="n">
-        <v>46234</v>
+        <v>46230</v>
       </c>
       <c r="G9" s="2" t="n">
         <v>46265</v>
@@ -850,7 +850,7 @@
         </is>
       </c>
       <c r="F10" s="2" t="n">
-        <v>46234</v>
+        <v>46230</v>
       </c>
       <c r="G10" s="2" t="n">
         <v>46265</v>
@@ -887,7 +887,7 @@
         </is>
       </c>
       <c r="F11" s="2" t="n">
-        <v>46234</v>
+        <v>46230</v>
       </c>
       <c r="G11" s="2" t="n">
         <v>46265</v>
@@ -928,7 +928,7 @@
         </is>
       </c>
       <c r="F12" s="2" t="n">
-        <v>46234</v>
+        <v>46230</v>
       </c>
       <c r="G12" s="2" t="n">
         <v>46265</v>
@@ -965,7 +965,7 @@
         </is>
       </c>
       <c r="F13" s="2" t="n">
-        <v>46234</v>
+        <v>46230</v>
       </c>
       <c r="G13" s="2" t="n">
         <v>46265</v>
@@ -1002,7 +1002,7 @@
         </is>
       </c>
       <c r="F14" s="2" t="n">
-        <v>46234</v>
+        <v>46230</v>
       </c>
       <c r="G14" s="2" t="n">
         <v>46265</v>
@@ -1039,7 +1039,7 @@
         </is>
       </c>
       <c r="F15" s="2" t="n">
-        <v>46234</v>
+        <v>46230</v>
       </c>
       <c r="G15" s="2" t="n">
         <v>46265</v>
@@ -1076,7 +1076,7 @@
         </is>
       </c>
       <c r="F16" s="2" t="n">
-        <v>46234</v>
+        <v>46230</v>
       </c>
       <c r="G16" s="2" t="n">
         <v>46265</v>
@@ -1173,28 +1173,28 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>日期標示：各標的分頁的週／月／年資料，一律標該期「實際最後交易日」</t>
+          <t>日期與數值：各標的分頁的週／月／年資料，日期欄標該期「第一個交易日」，收盤價取該期「最後一個交易日」的值，成交量為整期加總（與雅虎財經的做法一致）</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>Dates: weekly/monthly/yearly rows in each ticker sheet use the actual last trading day of the period</t>
+          <t>Dates and values: the date is the FIRST trading day of the period; Close/Adj Close are from the LAST trading day; Volume is the period total (same convention as Yahoo Finance)</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>Combined 對齊：日資料以交易日；週資料以該週週五；月資料以月底；年資料以 12/31</t>
+          <t>Combined 對齊：日資料以交易日；週資料以該週週一；月資料以月初；年資料以 1/1</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>Combined alignment: daily = trading day; weekly = that week's Friday; monthly = month end; yearly = Dec 31</t>
+          <t>Combined alignment: daily = trading day; weekly = that week's Monday; monthly = first of the month; yearly = Jan 1</t>
         </is>
       </c>
     </row>
@@ -1229,14 +1229,14 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>Flag 註記：Partial 未完整 = 結束日落在週期中間，該期資料不完整（仍保留最後交易日的數字）</t>
+          <t>Flag 註記：Partial 未完整 = 結束日落在週期中間，該期資料不完整（收盤價取截至結束日最新的一天）</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>Flag: Partial = the end date falls inside the period; the period is incomplete (the last trading day's value is kept)</t>
+          <t>Flag: Partial = the end date falls inside the period; the period is incomplete (values are from the latest trading day up to the end date)</t>
         </is>
       </c>
     </row>
@@ -1304,7 +1304,7 @@
     </row>
     <row r="2">
       <c r="A2" s="2" t="n">
-        <v>46234</v>
+        <v>46230</v>
       </c>
       <c r="B2" s="4" t="n">
         <v>97.05</v>
@@ -1323,7 +1323,7 @@
     </row>
     <row r="3">
       <c r="A3" s="2" t="n">
-        <v>46241</v>
+        <v>46237</v>
       </c>
       <c r="B3" s="4" t="n">
         <v>97.2</v>
@@ -1338,7 +1338,7 @@
     </row>
     <row r="4">
       <c r="A4" s="2" t="n">
-        <v>46248</v>
+        <v>46244</v>
       </c>
       <c r="B4" s="4" t="n">
         <v>94.51000000000001</v>
@@ -1353,7 +1353,7 @@
     </row>
     <row r="5">
       <c r="A5" s="2" t="n">
-        <v>46255</v>
+        <v>46251</v>
       </c>
       <c r="B5" s="4" t="n">
         <v>95.75</v>
@@ -1368,7 +1368,7 @@
     </row>
     <row r="6">
       <c r="A6" s="2" t="n">
-        <v>46262</v>
+        <v>46258</v>
       </c>
       <c r="B6" s="4" t="n">
         <v>98.89</v>
@@ -1450,7 +1450,7 @@
     </row>
     <row r="2">
       <c r="A2" s="2" t="n">
-        <v>46234</v>
+        <v>46230</v>
       </c>
       <c r="B2" s="4" t="n">
         <v>327.05</v>
@@ -1469,7 +1469,7 @@
     </row>
     <row r="3">
       <c r="A3" s="2" t="n">
-        <v>46241</v>
+        <v>46237</v>
       </c>
       <c r="B3" s="4" t="n">
         <v>325.63</v>
@@ -1484,7 +1484,7 @@
     </row>
     <row r="4">
       <c r="A4" s="2" t="n">
-        <v>46248</v>
+        <v>46244</v>
       </c>
       <c r="B4" s="4" t="n">
         <v>317.39</v>
@@ -1499,7 +1499,7 @@
     </row>
     <row r="5">
       <c r="A5" s="2" t="n">
-        <v>46255</v>
+        <v>46251</v>
       </c>
       <c r="B5" s="4" t="n">
         <v>309.81</v>
@@ -1514,7 +1514,7 @@
     </row>
     <row r="6">
       <c r="A6" s="2" t="n">
-        <v>46262</v>
+        <v>46258</v>
       </c>
       <c r="B6" s="4" t="n">
         <v>301.69</v>
@@ -1596,7 +1596,7 @@
     </row>
     <row r="2">
       <c r="A2" s="2" t="n">
-        <v>46234</v>
+        <v>46230</v>
       </c>
       <c r="B2" s="4" t="n">
         <v>23.63</v>
@@ -1615,7 +1615,7 @@
     </row>
     <row r="3">
       <c r="A3" s="2" t="n">
-        <v>46241</v>
+        <v>46237</v>
       </c>
       <c r="B3" s="4" t="n">
         <v>23.12</v>
@@ -1630,7 +1630,7 @@
     </row>
     <row r="4">
       <c r="A4" s="2" t="n">
-        <v>46248</v>
+        <v>46244</v>
       </c>
       <c r="B4" s="4" t="n">
         <v>22.55</v>
@@ -1645,7 +1645,7 @@
     </row>
     <row r="5">
       <c r="A5" s="2" t="n">
-        <v>46255</v>
+        <v>46251</v>
       </c>
       <c r="B5" s="4" t="n">
         <v>23.07</v>
@@ -1660,7 +1660,7 @@
     </row>
     <row r="6">
       <c r="A6" s="2" t="n">
-        <v>46262</v>
+        <v>46258</v>
       </c>
       <c r="B6" s="4" t="n">
         <v>22.69</v>
@@ -1742,7 +1742,7 @@
     </row>
     <row r="2">
       <c r="A2" s="2" t="n">
-        <v>46234</v>
+        <v>46230</v>
       </c>
       <c r="B2" s="4" t="n">
         <v>4.7</v>
@@ -1761,7 +1761,7 @@
     </row>
     <row r="3">
       <c r="A3" s="2" t="n">
-        <v>46241</v>
+        <v>46237</v>
       </c>
       <c r="B3" s="4" t="n">
         <v>4.689</v>
@@ -1776,7 +1776,7 @@
     </row>
     <row r="4">
       <c r="A4" s="2" t="n">
-        <v>46248</v>
+        <v>46244</v>
       </c>
       <c r="B4" s="4" t="n">
         <v>4.647</v>
@@ -1791,7 +1791,7 @@
     </row>
     <row r="5">
       <c r="A5" s="2" t="n">
-        <v>46255</v>
+        <v>46251</v>
       </c>
       <c r="B5" s="4" t="n">
         <v>4.699</v>
@@ -1806,7 +1806,7 @@
     </row>
     <row r="6">
       <c r="A6" s="2" t="n">
-        <v>46262</v>
+        <v>46258</v>
       </c>
       <c r="B6" s="4" t="n">
         <v>4.64</v>
@@ -1888,7 +1888,7 @@
     </row>
     <row r="2">
       <c r="A2" s="2" t="n">
-        <v>46234</v>
+        <v>46230</v>
       </c>
       <c r="B2" s="4" t="n">
         <v>2417.14</v>
@@ -1907,7 +1907,7 @@
     </row>
     <row r="3">
       <c r="A3" s="2" t="n">
-        <v>46241</v>
+        <v>46237</v>
       </c>
       <c r="B3" s="4" t="n">
         <v>2420.44</v>
@@ -1922,7 +1922,7 @@
     </row>
     <row r="4">
       <c r="A4" s="2" t="n">
-        <v>46248</v>
+        <v>46244</v>
       </c>
       <c r="B4" s="4" t="n">
         <v>2380.25</v>
@@ -1937,7 +1937,7 @@
     </row>
     <row r="5">
       <c r="A5" s="2" t="n">
-        <v>46255</v>
+        <v>46251</v>
       </c>
       <c r="B5" s="4" t="n">
         <v>2436.27</v>
@@ -1952,7 +1952,7 @@
     </row>
     <row r="6">
       <c r="A6" s="2" t="n">
-        <v>46262</v>
+        <v>46258</v>
       </c>
       <c r="B6" s="4" t="n">
         <v>2491.55</v>
@@ -2034,7 +2034,7 @@
     </row>
     <row r="2">
       <c r="A2" s="2" t="n">
-        <v>46234</v>
+        <v>46230</v>
       </c>
       <c r="B2" s="4" t="n">
         <v>149.91</v>
@@ -2053,7 +2053,7 @@
     </row>
     <row r="3">
       <c r="A3" s="2" t="n">
-        <v>46241</v>
+        <v>46237</v>
       </c>
       <c r="B3" s="4" t="n">
         <v>153.76</v>
@@ -2068,7 +2068,7 @@
     </row>
     <row r="4">
       <c r="A4" s="2" t="n">
-        <v>46248</v>
+        <v>46244</v>
       </c>
       <c r="B4" s="4" t="n">
         <v>153.67</v>
@@ -2083,7 +2083,7 @@
     </row>
     <row r="5">
       <c r="A5" s="2" t="n">
-        <v>46255</v>
+        <v>46251</v>
       </c>
       <c r="B5" s="4" t="n">
         <v>150.95</v>
@@ -2098,7 +2098,7 @@
     </row>
     <row r="6">
       <c r="A6" s="2" t="n">
-        <v>46262</v>
+        <v>46258</v>
       </c>
       <c r="B6" s="4" t="n">
         <v>151.09</v>
@@ -2180,7 +2180,7 @@
     </row>
     <row r="2">
       <c r="A2" s="2" t="n">
-        <v>46234</v>
+        <v>46230</v>
       </c>
       <c r="B2" s="4" t="n">
         <v>230.19</v>
@@ -2199,7 +2199,7 @@
     </row>
     <row r="3">
       <c r="A3" s="2" t="n">
-        <v>46241</v>
+        <v>46237</v>
       </c>
       <c r="B3" s="4" t="n">
         <v>233.26</v>
@@ -2214,7 +2214,7 @@
     </row>
     <row r="4">
       <c r="A4" s="2" t="n">
-        <v>46248</v>
+        <v>46244</v>
       </c>
       <c r="B4" s="4" t="n">
         <v>232.05</v>
@@ -2229,7 +2229,7 @@
     </row>
     <row r="5">
       <c r="A5" s="2" t="n">
-        <v>46255</v>
+        <v>46251</v>
       </c>
       <c r="B5" s="4" t="n">
         <v>232.37</v>
@@ -2244,7 +2244,7 @@
     </row>
     <row r="6">
       <c r="A6" s="2" t="n">
-        <v>46262</v>
+        <v>46258</v>
       </c>
       <c r="B6" s="4" t="n">
         <v>237.63</v>
@@ -2326,7 +2326,7 @@
     </row>
     <row r="2">
       <c r="A2" s="2" t="n">
-        <v>46234</v>
+        <v>46230</v>
       </c>
       <c r="B2" s="4" t="n">
         <v>286.18</v>
@@ -2345,7 +2345,7 @@
     </row>
     <row r="3">
       <c r="A3" s="2" t="n">
-        <v>46241</v>
+        <v>46237</v>
       </c>
       <c r="B3" s="4" t="n">
         <v>289.73</v>
@@ -2360,7 +2360,7 @@
     </row>
     <row r="4">
       <c r="A4" s="2" t="n">
-        <v>46248</v>
+        <v>46244</v>
       </c>
       <c r="B4" s="4" t="n">
         <v>297.4</v>
@@ -2375,7 +2375,7 @@
     </row>
     <row r="5">
       <c r="A5" s="2" t="n">
-        <v>46255</v>
+        <v>46251</v>
       </c>
       <c r="B5" s="4" t="n">
         <v>302.67</v>
@@ -2390,7 +2390,7 @@
     </row>
     <row r="6">
       <c r="A6" s="2" t="n">
-        <v>46262</v>
+        <v>46258</v>
       </c>
       <c r="B6" s="4" t="n">
         <v>294.98</v>
@@ -2472,7 +2472,7 @@
     </row>
     <row r="2">
       <c r="A2" s="2" t="n">
-        <v>46234</v>
+        <v>46230</v>
       </c>
       <c r="B2" s="4" t="n">
         <v>117.23</v>
@@ -2491,7 +2491,7 @@
     </row>
     <row r="3">
       <c r="A3" s="2" t="n">
-        <v>46241</v>
+        <v>46237</v>
       </c>
       <c r="B3" s="4" t="n">
         <v>117.73</v>
@@ -2506,7 +2506,7 @@
     </row>
     <row r="4">
       <c r="A4" s="2" t="n">
-        <v>46248</v>
+        <v>46244</v>
       </c>
       <c r="B4" s="4" t="n">
         <v>116.28</v>
@@ -2521,7 +2521,7 @@
     </row>
     <row r="5">
       <c r="A5" s="2" t="n">
-        <v>46255</v>
+        <v>46251</v>
       </c>
       <c r="B5" s="4" t="n">
         <v>114.99</v>
@@ -2536,7 +2536,7 @@
     </row>
     <row r="6">
       <c r="A6" s="2" t="n">
-        <v>46262</v>
+        <v>46258</v>
       </c>
       <c r="B6" s="4" t="n">
         <v>116.46</v>
@@ -2690,7 +2690,7 @@
     </row>
     <row r="2">
       <c r="A2" s="2" t="n">
-        <v>46234</v>
+        <v>46230</v>
       </c>
       <c r="B2" s="4" t="n">
         <v>43409.11</v>
@@ -2745,7 +2745,7 @@
     </row>
     <row r="3">
       <c r="A3" s="2" t="n">
-        <v>46241</v>
+        <v>46237</v>
       </c>
       <c r="B3" s="4" t="n">
         <v>44245.47</v>
@@ -2796,7 +2796,7 @@
     </row>
     <row r="4">
       <c r="A4" s="2" t="n">
-        <v>46248</v>
+        <v>46244</v>
       </c>
       <c r="B4" s="4" t="n">
         <v>44127.66</v>
@@ -2845,7 +2845,7 @@
     </row>
     <row r="5">
       <c r="A5" s="2" t="n">
-        <v>46255</v>
+        <v>46251</v>
       </c>
       <c r="B5" s="4" t="n">
         <v>43546.48</v>
@@ -2896,7 +2896,7 @@
     </row>
     <row r="6">
       <c r="A6" s="2" t="n">
-        <v>46262</v>
+        <v>46258</v>
       </c>
       <c r="B6" s="4" t="n">
         <v>43687.25</v>
@@ -2947,7 +2947,7 @@
     </row>
     <row r="7">
       <c r="A7" s="2" t="n">
-        <v>46269</v>
+        <v>46265</v>
       </c>
       <c r="B7" s="4" t="n">
         <v>43526.52</v>
@@ -3122,7 +3122,7 @@
     </row>
     <row r="2">
       <c r="A2" s="2" t="n">
-        <v>46234</v>
+        <v>46230</v>
       </c>
       <c r="B2" s="4" t="n">
         <v>44070.16</v>
@@ -3177,7 +3177,7 @@
     </row>
     <row r="3">
       <c r="A3" s="2" t="n">
-        <v>46241</v>
+        <v>46237</v>
       </c>
       <c r="B3" s="4" t="n">
         <v>44919.26</v>
@@ -3228,7 +3228,7 @@
     </row>
     <row r="4">
       <c r="A4" s="2" t="n">
-        <v>46248</v>
+        <v>46244</v>
       </c>
       <c r="B4" s="4" t="n">
         <v>44799.65</v>
@@ -3277,7 +3277,7 @@
     </row>
     <row r="5">
       <c r="A5" s="2" t="n">
-        <v>46255</v>
+        <v>46251</v>
       </c>
       <c r="B5" s="4" t="n">
         <v>44209.62</v>
@@ -3328,7 +3328,7 @@
     </row>
     <row r="6">
       <c r="A6" s="2" t="n">
-        <v>46262</v>
+        <v>46258</v>
       </c>
       <c r="B6" s="4" t="n">
         <v>44352.54</v>
@@ -3379,7 +3379,7 @@
     </row>
     <row r="7">
       <c r="A7" s="2" t="n">
-        <v>46269</v>
+        <v>46265</v>
       </c>
       <c r="B7" s="4" t="n">
         <v>44189.36</v>
@@ -3482,7 +3482,7 @@
     </row>
     <row r="2">
       <c r="A2" s="2" t="n">
-        <v>46234</v>
+        <v>46230</v>
       </c>
       <c r="B2" s="4" t="n">
         <v>44070.16</v>
@@ -3501,7 +3501,7 @@
     </row>
     <row r="3">
       <c r="A3" s="2" t="n">
-        <v>46241</v>
+        <v>46237</v>
       </c>
       <c r="B3" s="4" t="n">
         <v>44919.26</v>
@@ -3516,7 +3516,7 @@
     </row>
     <row r="4">
       <c r="A4" s="2" t="n">
-        <v>46248</v>
+        <v>46244</v>
       </c>
       <c r="B4" s="4" t="n">
         <v>44799.65</v>
@@ -3531,7 +3531,7 @@
     </row>
     <row r="5">
       <c r="A5" s="2" t="n">
-        <v>46254</v>
+        <v>46252</v>
       </c>
       <c r="B5" s="4" t="n">
         <v>44209.62</v>
@@ -3546,7 +3546,7 @@
     </row>
     <row r="6">
       <c r="A6" s="2" t="n">
-        <v>46262</v>
+        <v>46258</v>
       </c>
       <c r="B6" s="4" t="n">
         <v>44352.54</v>
@@ -3628,7 +3628,7 @@
     </row>
     <row r="2">
       <c r="A2" s="2" t="n">
-        <v>46234</v>
+        <v>46230</v>
       </c>
       <c r="B2" s="4" t="n">
         <v>39149.35</v>
@@ -3647,7 +3647,7 @@
     </row>
     <row r="3">
       <c r="A3" s="2" t="n">
-        <v>46241</v>
+        <v>46237</v>
       </c>
       <c r="B3" s="4" t="n">
         <v>40131.34</v>
@@ -3662,7 +3662,7 @@
     </row>
     <row r="4">
       <c r="A4" s="2" t="n">
-        <v>46255</v>
+        <v>46251</v>
       </c>
       <c r="B4" s="4" t="n">
         <v>40370.57</v>
@@ -3677,7 +3677,7 @@
     </row>
     <row r="5">
       <c r="A5" s="2" t="n">
-        <v>46262</v>
+        <v>46258</v>
       </c>
       <c r="B5" s="4" t="n">
         <v>40459.52</v>
@@ -3759,7 +3759,7 @@
     </row>
     <row r="2">
       <c r="A2" s="2" t="n">
-        <v>46234</v>
+        <v>46230</v>
       </c>
       <c r="B2" s="4" t="n">
         <v>768.95</v>
@@ -3778,7 +3778,7 @@
     </row>
     <row r="3">
       <c r="A3" s="2" t="n">
-        <v>46241</v>
+        <v>46237</v>
       </c>
       <c r="B3" s="4" t="n">
         <v>750.46</v>
@@ -3793,7 +3793,7 @@
     </row>
     <row r="4">
       <c r="A4" s="2" t="n">
-        <v>46248</v>
+        <v>46244</v>
       </c>
       <c r="B4" s="4" t="n">
         <v>768.7</v>
@@ -3808,7 +3808,7 @@
     </row>
     <row r="5">
       <c r="A5" s="2" t="n">
-        <v>46255</v>
+        <v>46251</v>
       </c>
       <c r="B5" s="4" t="n">
         <v>758.21</v>
@@ -3823,7 +3823,7 @@
     </row>
     <row r="6">
       <c r="A6" s="2" t="n">
-        <v>46262</v>
+        <v>46258</v>
       </c>
       <c r="B6" s="4" t="n">
         <v>765.37</v>
@@ -3905,7 +3905,7 @@
     </row>
     <row r="2">
       <c r="A2" s="2" t="n">
-        <v>46234</v>
+        <v>46230</v>
       </c>
       <c r="B2" s="4" t="n">
         <v>68.98</v>
@@ -3924,7 +3924,7 @@
     </row>
     <row r="3">
       <c r="A3" s="2" t="n">
-        <v>46241</v>
+        <v>46237</v>
       </c>
       <c r="B3" s="4" t="n">
         <v>67.5</v>
@@ -3939,7 +3939,7 @@
     </row>
     <row r="4">
       <c r="A4" s="2" t="n">
-        <v>46248</v>
+        <v>46244</v>
       </c>
       <c r="B4" s="4" t="n">
         <v>67.55</v>
@@ -3954,7 +3954,7 @@
     </row>
     <row r="5">
       <c r="A5" s="2" t="n">
-        <v>46255</v>
+        <v>46251</v>
       </c>
       <c r="B5" s="4" t="n">
         <v>65.81</v>
@@ -3969,7 +3969,7 @@
     </row>
     <row r="6">
       <c r="A6" s="2" t="n">
-        <v>46262</v>
+        <v>46258</v>
       </c>
       <c r="B6" s="4" t="n">
         <v>67.73</v>
@@ -4051,7 +4051,7 @@
     </row>
     <row r="2">
       <c r="A2" s="2" t="n">
-        <v>46234</v>
+        <v>46230</v>
       </c>
       <c r="B2" s="4" t="n">
         <v>54.19</v>
@@ -4070,7 +4070,7 @@
     </row>
     <row r="3">
       <c r="A3" s="2" t="n">
-        <v>46241</v>
+        <v>46237</v>
       </c>
       <c r="B3" s="4" t="n">
         <v>55.11</v>
@@ -4085,7 +4085,7 @@
     </row>
     <row r="4">
       <c r="A4" s="2" t="n">
-        <v>46248</v>
+        <v>46244</v>
       </c>
       <c r="B4" s="4" t="n">
         <v>54.01</v>
@@ -4100,7 +4100,7 @@
     </row>
     <row r="5">
       <c r="A5" s="2" t="n">
-        <v>46255</v>
+        <v>46251</v>
       </c>
       <c r="B5" s="4" t="n">
         <v>52.46</v>
@@ -4115,7 +4115,7 @@
     </row>
     <row r="6">
       <c r="A6" s="2" t="n">
-        <v>46262</v>
+        <v>46258</v>
       </c>
       <c r="B6" s="4" t="n">
         <v>54.02</v>
@@ -4197,7 +4197,7 @@
     </row>
     <row r="2">
       <c r="A2" s="2" t="n">
-        <v>46234</v>
+        <v>46230</v>
       </c>
       <c r="B2" s="4" t="n">
         <v>111.15</v>
@@ -4216,7 +4216,7 @@
     </row>
     <row r="3">
       <c r="A3" s="2" t="n">
-        <v>46241</v>
+        <v>46237</v>
       </c>
       <c r="B3" s="4" t="n">
         <v>113.56</v>
@@ -4231,7 +4231,7 @@
     </row>
     <row r="4">
       <c r="A4" s="2" t="n">
-        <v>46248</v>
+        <v>46244</v>
       </c>
       <c r="B4" s="4" t="n">
         <v>116.97</v>
@@ -4246,7 +4246,7 @@
     </row>
     <row r="5">
       <c r="A5" s="2" t="n">
-        <v>46255</v>
+        <v>46251</v>
       </c>
       <c r="B5" s="4" t="n">
         <v>119.85</v>
@@ -4261,7 +4261,7 @@
     </row>
     <row r="6">
       <c r="A6" s="2" t="n">
-        <v>46262</v>
+        <v>46258</v>
       </c>
       <c r="B6" s="4" t="n">
         <v>121.31</v>

</xml_diff>

<commit_message>
Show Period and Trade Date columns and share rows across all sheets
Per-ticker sheets now carry the alignment date and the actual value date,
and list the same rows as Combined, leaving closed periods blank.

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/sample/PortfolioData_W_20260803_20260831_SAMPLE.xlsx
+++ b/sample/PortfolioData_W_20260803_20260831_SAMPLE.xlsx
@@ -458,7 +458,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I41"/>
+  <dimension ref="A1:I47"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -500,17 +500,17 @@
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
-          <t>第一筆日期 First Date</t>
+          <t>第一筆取值日 First Trade Date</t>
         </is>
       </c>
       <c r="G1" s="1" t="inlineStr">
         <is>
-          <t>最後一筆日期 Last Date</t>
+          <t>最後一筆取值日 Last Trade Date</t>
         </is>
       </c>
       <c r="H1" s="1" t="inlineStr">
         <is>
-          <t>筆數 Rows</t>
+          <t>有資料筆數 Rows</t>
         </is>
       </c>
       <c r="I1" s="1" t="inlineStr">
@@ -546,7 +546,7 @@
         </is>
       </c>
       <c r="F2" s="2" t="n">
-        <v>46230</v>
+        <v>46234</v>
       </c>
       <c r="G2" s="2" t="n">
         <v>46265</v>
@@ -556,7 +556,7 @@
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>示範：2026-08-17 該週週一休市，日期欄標 08-18（第一個交易日），Combined 仍在 08-17 / demo: Monday closed, date is 08-18, Combined stays at 08-17</t>
+          <t>示範：2026-08-17 該週週五休市，取值日為 08-20 / demo: Friday closed, Trade Date is 08-20</t>
         </is>
       </c>
     </row>
@@ -587,7 +587,7 @@
         </is>
       </c>
       <c r="F3" s="2" t="n">
-        <v>46230</v>
+        <v>46234</v>
       </c>
       <c r="G3" s="2" t="n">
         <v>46265</v>
@@ -597,7 +597,7 @@
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>示範：2026-08-10 該週整週休市，Combined 留白 / demo: whole week closed, blank in Combined</t>
+          <t>示範：2026-08-10 該週整週休市，該列留白並標休市 / demo: whole week closed, row is blank and flagged</t>
         </is>
       </c>
     </row>
@@ -628,7 +628,7 @@
         </is>
       </c>
       <c r="F4" s="2" t="n">
-        <v>46230</v>
+        <v>46234</v>
       </c>
       <c r="G4" s="2" t="n">
         <v>46265</v>
@@ -665,7 +665,7 @@
         </is>
       </c>
       <c r="F5" s="2" t="n">
-        <v>46230</v>
+        <v>46234</v>
       </c>
       <c r="G5" s="2" t="n">
         <v>46265</v>
@@ -702,7 +702,7 @@
         </is>
       </c>
       <c r="F6" s="2" t="n">
-        <v>46230</v>
+        <v>46234</v>
       </c>
       <c r="G6" s="2" t="n">
         <v>46265</v>
@@ -739,7 +739,7 @@
         </is>
       </c>
       <c r="F7" s="2" t="n">
-        <v>46230</v>
+        <v>46234</v>
       </c>
       <c r="G7" s="2" t="n">
         <v>46265</v>
@@ -776,7 +776,7 @@
         </is>
       </c>
       <c r="F8" s="2" t="n">
-        <v>46230</v>
+        <v>46234</v>
       </c>
       <c r="G8" s="2" t="n">
         <v>46265</v>
@@ -813,7 +813,7 @@
         </is>
       </c>
       <c r="F9" s="2" t="n">
-        <v>46230</v>
+        <v>46234</v>
       </c>
       <c r="G9" s="2" t="n">
         <v>46265</v>
@@ -850,7 +850,7 @@
         </is>
       </c>
       <c r="F10" s="2" t="n">
-        <v>46230</v>
+        <v>46234</v>
       </c>
       <c r="G10" s="2" t="n">
         <v>46265</v>
@@ -887,7 +887,7 @@
         </is>
       </c>
       <c r="F11" s="2" t="n">
-        <v>46230</v>
+        <v>46234</v>
       </c>
       <c r="G11" s="2" t="n">
         <v>46265</v>
@@ -928,7 +928,7 @@
         </is>
       </c>
       <c r="F12" s="2" t="n">
-        <v>46230</v>
+        <v>46234</v>
       </c>
       <c r="G12" s="2" t="n">
         <v>46265</v>
@@ -965,7 +965,7 @@
         </is>
       </c>
       <c r="F13" s="2" t="n">
-        <v>46230</v>
+        <v>46234</v>
       </c>
       <c r="G13" s="2" t="n">
         <v>46265</v>
@@ -1002,7 +1002,7 @@
         </is>
       </c>
       <c r="F14" s="2" t="n">
-        <v>46230</v>
+        <v>46234</v>
       </c>
       <c r="G14" s="2" t="n">
         <v>46265</v>
@@ -1039,7 +1039,7 @@
         </is>
       </c>
       <c r="F15" s="2" t="n">
-        <v>46230</v>
+        <v>46234</v>
       </c>
       <c r="G15" s="2" t="n">
         <v>46265</v>
@@ -1076,7 +1076,7 @@
         </is>
       </c>
       <c r="F16" s="2" t="n">
-        <v>46230</v>
+        <v>46234</v>
       </c>
       <c r="G16" s="2" t="n">
         <v>46265</v>
@@ -1173,82 +1173,124 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>日期與數值：各標的分頁的週／月／年資料，日期欄標該期「第一個交易日」，收盤價取該期「最後一個交易日」的值，成交量為整期加總（與雅虎財經的做法一致）</t>
+          <t>兩個日期欄：Period 期間 = 對齊日（日資料為當天、週資料為該週週一、月資料為該月 1 日、年資料為 1/1，與雅虎財經的日期標示相同），所有標的分頁與 Combined 分頁都一樣；Trade Date 取值日 = 收盤價實際來自哪一天（該期最後一個交易日；結束日落在期中時，為截至結束日最新的一天）</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>Dates and values: the date is the FIRST trading day of the period; Close/Adj Close are from the LAST trading day; Volume is the period total (same convention as Yahoo Finance)</t>
+          <t>Two date columns: Period = alignment date (that week's Monday, the 1st of the month, Jan 1, or the day itself for daily data), identical in every sheet; Trade Date = the day Close/Adj Close actually come from (the last trading day of the period)</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>Combined 對齊：日資料以交易日；週資料以該週週一；月資料以月初；年資料以 1/1</t>
+          <t>收盤價與調整後收盤價取該期最後一個交易日的值，成交量為整期加總</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>Combined alignment: daily = trading day; weekly = that week's Monday; monthly = first of the month; yearly = Jan 1</t>
+          <t>Close and Adj Close are from the last trading day of the period; Volume is the total over the period</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>Combined 留白：該期該市場沒有交易時，儲存格為空白，不補值。計算共變異數前請自行處理</t>
+          <t>Combined 對齊：日資料以交易日；週資料以該週週一；月資料以月初；年資料以 1/1</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>Combined blanks: a cell is empty when that market has no data for the period; handle before computing covariances</t>
+          <t>Combined alignment: daily = trading day; weekly = that week's Monday; monthly = first of the month; yearly = Jan 1</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>Flag 註記：Prior period 前一期 = 起始日之前多抓的一期，供計算第一期報酬</t>
+          <t>所有分頁的列相同：列 = 所有已下載標的的期間聯集。某標的該期沒有交易時，該列只填 Period，取值日與數值留白，Flag 標 No trading 休市；標的尚未有資料的期間標 No data 無資料。所有標的都沒有交易的期間不會出現</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>Flag: Prior period = one extra period before the start date, for computing the first return</t>
+          <t>All sheets share the same rows (union of periods). When a ticker has no trading in a period, only Period is filled, Trade Date and values are blank, and Flag says No trading; earlier periods are flagged No data</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>Flag 註記：Partial 未完整 = 結束日落在週期中間，該期資料不完整（收盤價取截至結束日最新的一天）</t>
+          <t>空白格不補值。以公式計算報酬或共變異數前，請自行處理（例如以 Flag 篩選掉空白列）</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>Flag: Partial = the end date falls inside the period; the period is incomplete (values are from the latest trading day up to the end date)</t>
+          <t>Blank cells are not filled. Handle them yourself (e.g. filter out blank rows using Flag) before computing returns or covariances</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>Flag 註記：Intraday 盤中 = 日資料最後一筆為當日尚未收盤的盤中價</t>
+          <t>Flag 註記：No trading 休市 = 該標的在該期沒有交易；No data 無資料 = 該標的在該期之前尚無資料</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
+        <is>
+          <t>Flag: No trading = the ticker has no trading in that period; No data = no data before this period</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>Flag 註記：Prior period 前一期 = 起始日之前多抓的一期，供計算第一期報酬</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>Flag: Prior period = one extra period before the start date, for computing the first return</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>Flag 註記：Partial 未完整 = 結束日落在週期中間，該期資料不完整（收盤價取截至結束日最新的一天）</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>Flag: Partial = the end date falls inside the period; the period is incomplete (values are from the latest trading day up to the end date)</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>Flag 註記：Intraday 盤中 = 日資料最後一筆為當日尚未收盤的盤中價</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
         <is>
           <t>Flag: Intraday = the last daily row is an unfinished intraday price</t>
         </is>
@@ -1265,38 +1307,44 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E7"/>
+  <dimension ref="A1:F7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
-    <col width="16" customWidth="1" min="2" max="2"/>
-    <col width="22" customWidth="1" min="3" max="3"/>
-    <col width="16" customWidth="1" min="4" max="4"/>
-    <col width="20" customWidth="1" min="5" max="5"/>
+    <col width="15" customWidth="1" min="2" max="2"/>
+    <col width="16" customWidth="1" min="3" max="3"/>
+    <col width="24" customWidth="1" min="4" max="4"/>
+    <col width="16" customWidth="1" min="5" max="5"/>
+    <col width="22" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1" ht="32" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Date 日期</t>
+          <t>Period 期間</t>
         </is>
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
+          <t>Trade Date 取值日</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
           <t>Close 收盤價</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>Adj Close 調整後收盤價</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>Volume 成交量</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>Flag 註記</t>
         </is>
@@ -1306,16 +1354,19 @@
       <c r="A2" s="2" t="n">
         <v>46230</v>
       </c>
-      <c r="B2" s="4" t="n">
+      <c r="B2" s="2" t="n">
+        <v>46234</v>
+      </c>
+      <c r="C2" s="4" t="n">
         <v>97.05</v>
       </c>
-      <c r="C2" s="4" t="n">
+      <c r="D2" s="4" t="n">
         <v>95.59</v>
       </c>
-      <c r="D2" s="5" t="n">
+      <c r="E2" s="5" t="n">
         <v>12813867</v>
       </c>
-      <c r="E2" t="inlineStr">
+      <c r="F2" t="inlineStr">
         <is>
           <t>Prior period 前一期</t>
         </is>
@@ -1325,76 +1376,91 @@
       <c r="A3" s="2" t="n">
         <v>46237</v>
       </c>
-      <c r="B3" s="4" t="n">
+      <c r="B3" s="2" t="n">
+        <v>46241</v>
+      </c>
+      <c r="C3" s="4" t="n">
         <v>97.2</v>
       </c>
-      <c r="C3" s="4" t="n">
+      <c r="D3" s="4" t="n">
         <v>95.73999999999999</v>
       </c>
-      <c r="D3" s="5" t="n">
+      <c r="E3" s="5" t="n">
         <v>37114241</v>
       </c>
-      <c r="E3" t="inlineStr"/>
+      <c r="F3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" s="2" t="n">
         <v>46244</v>
       </c>
-      <c r="B4" s="4" t="n">
+      <c r="B4" s="2" t="n">
+        <v>46248</v>
+      </c>
+      <c r="C4" s="4" t="n">
         <v>94.51000000000001</v>
       </c>
-      <c r="C4" s="4" t="n">
+      <c r="D4" s="4" t="n">
         <v>93.09</v>
       </c>
-      <c r="D4" s="5" t="n">
+      <c r="E4" s="5" t="n">
         <v>21539150</v>
       </c>
-      <c r="E4" t="inlineStr"/>
+      <c r="F4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" s="2" t="n">
         <v>46251</v>
       </c>
-      <c r="B5" s="4" t="n">
+      <c r="B5" s="2" t="n">
+        <v>46255</v>
+      </c>
+      <c r="C5" s="4" t="n">
         <v>95.75</v>
       </c>
-      <c r="C5" s="4" t="n">
+      <c r="D5" s="4" t="n">
         <v>94.31</v>
       </c>
-      <c r="D5" s="5" t="n">
+      <c r="E5" s="5" t="n">
         <v>65116457</v>
       </c>
-      <c r="E5" t="inlineStr"/>
+      <c r="F5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" s="2" t="n">
         <v>46258</v>
       </c>
-      <c r="B6" s="4" t="n">
+      <c r="B6" s="2" t="n">
+        <v>46262</v>
+      </c>
+      <c r="C6" s="4" t="n">
         <v>98.89</v>
       </c>
-      <c r="C6" s="4" t="n">
+      <c r="D6" s="4" t="n">
         <v>97.41</v>
       </c>
-      <c r="D6" s="5" t="n">
+      <c r="E6" s="5" t="n">
         <v>52084737</v>
       </c>
-      <c r="E6" t="inlineStr"/>
+      <c r="F6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" s="2" t="n">
         <v>46265</v>
       </c>
-      <c r="B7" s="4" t="n">
+      <c r="B7" s="2" t="n">
+        <v>46265</v>
+      </c>
+      <c r="C7" s="4" t="n">
         <v>97.97</v>
       </c>
-      <c r="C7" s="4" t="n">
+      <c r="D7" s="4" t="n">
         <v>96.5</v>
       </c>
-      <c r="D7" s="5" t="n">
+      <c r="E7" s="5" t="n">
         <v>4937999</v>
       </c>
-      <c r="E7" t="inlineStr">
+      <c r="F7" t="inlineStr">
         <is>
           <t>Partial 未完整</t>
         </is>
@@ -1411,38 +1477,44 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E7"/>
+  <dimension ref="A1:F7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
-    <col width="16" customWidth="1" min="2" max="2"/>
-    <col width="22" customWidth="1" min="3" max="3"/>
-    <col width="16" customWidth="1" min="4" max="4"/>
-    <col width="20" customWidth="1" min="5" max="5"/>
+    <col width="15" customWidth="1" min="2" max="2"/>
+    <col width="16" customWidth="1" min="3" max="3"/>
+    <col width="24" customWidth="1" min="4" max="4"/>
+    <col width="16" customWidth="1" min="5" max="5"/>
+    <col width="22" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1" ht="32" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Date 日期</t>
+          <t>Period 期間</t>
         </is>
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
+          <t>Trade Date 取值日</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
           <t>Close 收盤價</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>Adj Close 調整後收盤價</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>Volume 成交量</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>Flag 註記</t>
         </is>
@@ -1452,16 +1524,19 @@
       <c r="A2" s="2" t="n">
         <v>46230</v>
       </c>
-      <c r="B2" s="4" t="n">
+      <c r="B2" s="2" t="n">
+        <v>46234</v>
+      </c>
+      <c r="C2" s="4" t="n">
         <v>327.05</v>
       </c>
-      <c r="C2" s="4" t="n">
+      <c r="D2" s="4" t="n">
         <v>322.14</v>
       </c>
-      <c r="D2" s="5" t="n">
+      <c r="E2" s="5" t="n">
         <v>22246633</v>
       </c>
-      <c r="E2" t="inlineStr">
+      <c r="F2" t="inlineStr">
         <is>
           <t>Prior period 前一期</t>
         </is>
@@ -1471,76 +1546,91 @@
       <c r="A3" s="2" t="n">
         <v>46237</v>
       </c>
-      <c r="B3" s="4" t="n">
+      <c r="B3" s="2" t="n">
+        <v>46241</v>
+      </c>
+      <c r="C3" s="4" t="n">
         <v>325.63</v>
       </c>
-      <c r="C3" s="4" t="n">
+      <c r="D3" s="4" t="n">
         <v>320.75</v>
       </c>
-      <c r="D3" s="5" t="n">
+      <c r="E3" s="5" t="n">
         <v>8480894</v>
       </c>
-      <c r="E3" t="inlineStr"/>
+      <c r="F3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" s="2" t="n">
         <v>46244</v>
       </c>
-      <c r="B4" s="4" t="n">
+      <c r="B4" s="2" t="n">
+        <v>46248</v>
+      </c>
+      <c r="C4" s="4" t="n">
         <v>317.39</v>
       </c>
-      <c r="C4" s="4" t="n">
+      <c r="D4" s="4" t="n">
         <v>312.63</v>
       </c>
-      <c r="D4" s="5" t="n">
+      <c r="E4" s="5" t="n">
         <v>73924865</v>
       </c>
-      <c r="E4" t="inlineStr"/>
+      <c r="F4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" s="2" t="n">
         <v>46251</v>
       </c>
-      <c r="B5" s="4" t="n">
+      <c r="B5" s="2" t="n">
+        <v>46255</v>
+      </c>
+      <c r="C5" s="4" t="n">
         <v>309.81</v>
       </c>
-      <c r="C5" s="4" t="n">
+      <c r="D5" s="4" t="n">
         <v>305.16</v>
       </c>
-      <c r="D5" s="5" t="n">
+      <c r="E5" s="5" t="n">
         <v>80220482</v>
       </c>
-      <c r="E5" t="inlineStr"/>
+      <c r="F5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" s="2" t="n">
         <v>46258</v>
       </c>
-      <c r="B6" s="4" t="n">
+      <c r="B6" s="2" t="n">
+        <v>46262</v>
+      </c>
+      <c r="C6" s="4" t="n">
         <v>301.69</v>
       </c>
-      <c r="C6" s="4" t="n">
+      <c r="D6" s="4" t="n">
         <v>297.16</v>
       </c>
-      <c r="D6" s="5" t="n">
+      <c r="E6" s="5" t="n">
         <v>70106871</v>
       </c>
-      <c r="E6" t="inlineStr"/>
+      <c r="F6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" s="2" t="n">
         <v>46265</v>
       </c>
-      <c r="B7" s="4" t="n">
+      <c r="B7" s="2" t="n">
+        <v>46265</v>
+      </c>
+      <c r="C7" s="4" t="n">
         <v>296.85</v>
       </c>
-      <c r="C7" s="4" t="n">
+      <c r="D7" s="4" t="n">
         <v>292.4</v>
       </c>
-      <c r="D7" s="5" t="n">
+      <c r="E7" s="5" t="n">
         <v>13535642</v>
       </c>
-      <c r="E7" t="inlineStr">
+      <c r="F7" t="inlineStr">
         <is>
           <t>Partial 未完整</t>
         </is>
@@ -1557,38 +1647,44 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E7"/>
+  <dimension ref="A1:F7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
-    <col width="16" customWidth="1" min="2" max="2"/>
-    <col width="22" customWidth="1" min="3" max="3"/>
-    <col width="16" customWidth="1" min="4" max="4"/>
-    <col width="20" customWidth="1" min="5" max="5"/>
+    <col width="15" customWidth="1" min="2" max="2"/>
+    <col width="16" customWidth="1" min="3" max="3"/>
+    <col width="24" customWidth="1" min="4" max="4"/>
+    <col width="16" customWidth="1" min="5" max="5"/>
+    <col width="22" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1" ht="32" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Date 日期</t>
+          <t>Period 期間</t>
         </is>
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
+          <t>Trade Date 取值日</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
           <t>Close 收盤價</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>Adj Close 調整後收盤價</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>Volume 成交量</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>Flag 註記</t>
         </is>
@@ -1598,16 +1694,19 @@
       <c r="A2" s="2" t="n">
         <v>46230</v>
       </c>
-      <c r="B2" s="4" t="n">
+      <c r="B2" s="2" t="n">
+        <v>46234</v>
+      </c>
+      <c r="C2" s="4" t="n">
         <v>23.63</v>
       </c>
-      <c r="C2" s="4" t="n">
+      <c r="D2" s="4" t="n">
         <v>23.28</v>
       </c>
-      <c r="D2" s="5" t="n">
+      <c r="E2" s="5" t="n">
         <v>52381235</v>
       </c>
-      <c r="E2" t="inlineStr">
+      <c r="F2" t="inlineStr">
         <is>
           <t>Prior period 前一期</t>
         </is>
@@ -1617,76 +1716,91 @@
       <c r="A3" s="2" t="n">
         <v>46237</v>
       </c>
-      <c r="B3" s="4" t="n">
+      <c r="B3" s="2" t="n">
+        <v>46241</v>
+      </c>
+      <c r="C3" s="4" t="n">
         <v>23.12</v>
       </c>
-      <c r="C3" s="4" t="n">
+      <c r="D3" s="4" t="n">
         <v>22.77</v>
       </c>
-      <c r="D3" s="5" t="n">
+      <c r="E3" s="5" t="n">
         <v>7875845</v>
       </c>
-      <c r="E3" t="inlineStr"/>
+      <c r="F3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" s="2" t="n">
         <v>46244</v>
       </c>
-      <c r="B4" s="4" t="n">
+      <c r="B4" s="2" t="n">
+        <v>46248</v>
+      </c>
+      <c r="C4" s="4" t="n">
         <v>22.55</v>
       </c>
-      <c r="C4" s="4" t="n">
+      <c r="D4" s="4" t="n">
         <v>22.21</v>
       </c>
-      <c r="D4" s="5" t="n">
+      <c r="E4" s="5" t="n">
         <v>35210966</v>
       </c>
-      <c r="E4" t="inlineStr"/>
+      <c r="F4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" s="2" t="n">
         <v>46251</v>
       </c>
-      <c r="B5" s="4" t="n">
+      <c r="B5" s="2" t="n">
+        <v>46255</v>
+      </c>
+      <c r="C5" s="4" t="n">
         <v>23.07</v>
       </c>
-      <c r="C5" s="4" t="n">
+      <c r="D5" s="4" t="n">
         <v>22.72</v>
       </c>
-      <c r="D5" s="5" t="n">
+      <c r="E5" s="5" t="n">
         <v>69962541</v>
       </c>
-      <c r="E5" t="inlineStr"/>
+      <c r="F5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" s="2" t="n">
         <v>46258</v>
       </c>
-      <c r="B6" s="4" t="n">
+      <c r="B6" s="2" t="n">
+        <v>46262</v>
+      </c>
+      <c r="C6" s="4" t="n">
         <v>22.69</v>
       </c>
-      <c r="C6" s="4" t="n">
+      <c r="D6" s="4" t="n">
         <v>22.35</v>
       </c>
-      <c r="D6" s="5" t="n">
+      <c r="E6" s="5" t="n">
         <v>88150123</v>
       </c>
-      <c r="E6" t="inlineStr"/>
+      <c r="F6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" s="2" t="n">
         <v>46265</v>
       </c>
-      <c r="B7" s="4" t="n">
+      <c r="B7" s="2" t="n">
+        <v>46265</v>
+      </c>
+      <c r="C7" s="4" t="n">
         <v>22.05</v>
       </c>
-      <c r="C7" s="4" t="n">
+      <c r="D7" s="4" t="n">
         <v>21.72</v>
       </c>
-      <c r="D7" s="5" t="n">
+      <c r="E7" s="5" t="n">
         <v>67417999</v>
       </c>
-      <c r="E7" t="inlineStr">
+      <c r="F7" t="inlineStr">
         <is>
           <t>Partial 未完整</t>
         </is>
@@ -1703,38 +1817,44 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E7"/>
+  <dimension ref="A1:F7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
-    <col width="16" customWidth="1" min="2" max="2"/>
-    <col width="22" customWidth="1" min="3" max="3"/>
-    <col width="16" customWidth="1" min="4" max="4"/>
-    <col width="20" customWidth="1" min="5" max="5"/>
+    <col width="15" customWidth="1" min="2" max="2"/>
+    <col width="16" customWidth="1" min="3" max="3"/>
+    <col width="24" customWidth="1" min="4" max="4"/>
+    <col width="16" customWidth="1" min="5" max="5"/>
+    <col width="22" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1" ht="32" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Date 日期</t>
+          <t>Period 期間</t>
         </is>
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
+          <t>Trade Date 取值日</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
           <t>Yield (%) 殖利率</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>Adj Yield (%) 調整後殖利率</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>Volume 成交量</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>Flag 註記</t>
         </is>
@@ -1744,16 +1864,19 @@
       <c r="A2" s="2" t="n">
         <v>46230</v>
       </c>
-      <c r="B2" s="4" t="n">
-        <v>4.7</v>
+      <c r="B2" s="2" t="n">
+        <v>46234</v>
       </c>
       <c r="C2" s="4" t="n">
         <v>4.7</v>
       </c>
-      <c r="D2" s="5" t="n">
+      <c r="D2" s="4" t="n">
+        <v>4.7</v>
+      </c>
+      <c r="E2" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="E2" t="inlineStr">
+      <c r="F2" t="inlineStr">
         <is>
           <t>Prior period 前一期</t>
         </is>
@@ -1763,76 +1886,91 @@
       <c r="A3" s="2" t="n">
         <v>46237</v>
       </c>
-      <c r="B3" s="4" t="n">
-        <v>4.689</v>
+      <c r="B3" s="2" t="n">
+        <v>46241</v>
       </c>
       <c r="C3" s="4" t="n">
         <v>4.689</v>
       </c>
-      <c r="D3" s="5" t="n">
+      <c r="D3" s="4" t="n">
+        <v>4.689</v>
+      </c>
+      <c r="E3" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="E3" t="inlineStr"/>
+      <c r="F3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" s="2" t="n">
         <v>46244</v>
       </c>
-      <c r="B4" s="4" t="n">
-        <v>4.647</v>
+      <c r="B4" s="2" t="n">
+        <v>46248</v>
       </c>
       <c r="C4" s="4" t="n">
         <v>4.647</v>
       </c>
-      <c r="D4" s="5" t="n">
+      <c r="D4" s="4" t="n">
+        <v>4.647</v>
+      </c>
+      <c r="E4" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="E4" t="inlineStr"/>
+      <c r="F4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" s="2" t="n">
         <v>46251</v>
       </c>
-      <c r="B5" s="4" t="n">
-        <v>4.699</v>
+      <c r="B5" s="2" t="n">
+        <v>46255</v>
       </c>
       <c r="C5" s="4" t="n">
         <v>4.699</v>
       </c>
-      <c r="D5" s="5" t="n">
+      <c r="D5" s="4" t="n">
+        <v>4.699</v>
+      </c>
+      <c r="E5" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="E5" t="inlineStr"/>
+      <c r="F5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" s="2" t="n">
         <v>46258</v>
       </c>
-      <c r="B6" s="4" t="n">
-        <v>4.64</v>
+      <c r="B6" s="2" t="n">
+        <v>46262</v>
       </c>
       <c r="C6" s="4" t="n">
         <v>4.64</v>
       </c>
-      <c r="D6" s="5" t="n">
+      <c r="D6" s="4" t="n">
+        <v>4.64</v>
+      </c>
+      <c r="E6" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="E6" t="inlineStr"/>
+      <c r="F6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" s="2" t="n">
         <v>46265</v>
       </c>
-      <c r="B7" s="4" t="n">
-        <v>4.646</v>
+      <c r="B7" s="2" t="n">
+        <v>46265</v>
       </c>
       <c r="C7" s="4" t="n">
         <v>4.646</v>
       </c>
-      <c r="D7" s="5" t="n">
+      <c r="D7" s="4" t="n">
+        <v>4.646</v>
+      </c>
+      <c r="E7" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="E7" t="inlineStr">
+      <c r="F7" t="inlineStr">
         <is>
           <t>Partial 未完整</t>
         </is>
@@ -1849,38 +1987,44 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E7"/>
+  <dimension ref="A1:F7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
-    <col width="16" customWidth="1" min="2" max="2"/>
-    <col width="22" customWidth="1" min="3" max="3"/>
-    <col width="16" customWidth="1" min="4" max="4"/>
-    <col width="20" customWidth="1" min="5" max="5"/>
+    <col width="15" customWidth="1" min="2" max="2"/>
+    <col width="16" customWidth="1" min="3" max="3"/>
+    <col width="24" customWidth="1" min="4" max="4"/>
+    <col width="16" customWidth="1" min="5" max="5"/>
+    <col width="22" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1" ht="32" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Date 日期</t>
+          <t>Period 期間</t>
         </is>
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
+          <t>Trade Date 取值日</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
           <t>Close 收盤價</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>Adj Close 調整後收盤價</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>Volume 成交量</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>Flag 註記</t>
         </is>
@@ -1890,16 +2034,19 @@
       <c r="A2" s="2" t="n">
         <v>46230</v>
       </c>
-      <c r="B2" s="4" t="n">
+      <c r="B2" s="2" t="n">
+        <v>46234</v>
+      </c>
+      <c r="C2" s="4" t="n">
         <v>2417.14</v>
       </c>
-      <c r="C2" s="4" t="n">
+      <c r="D2" s="4" t="n">
         <v>2380.88</v>
       </c>
-      <c r="D2" s="5" t="n">
+      <c r="E2" s="5" t="n">
         <v>59564514</v>
       </c>
-      <c r="E2" t="inlineStr">
+      <c r="F2" t="inlineStr">
         <is>
           <t>Prior period 前一期</t>
         </is>
@@ -1909,76 +2056,91 @@
       <c r="A3" s="2" t="n">
         <v>46237</v>
       </c>
-      <c r="B3" s="4" t="n">
+      <c r="B3" s="2" t="n">
+        <v>46241</v>
+      </c>
+      <c r="C3" s="4" t="n">
         <v>2420.44</v>
       </c>
-      <c r="C3" s="4" t="n">
+      <c r="D3" s="4" t="n">
         <v>2384.13</v>
       </c>
-      <c r="D3" s="5" t="n">
+      <c r="E3" s="5" t="n">
         <v>3990777</v>
       </c>
-      <c r="E3" t="inlineStr"/>
+      <c r="F3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" s="2" t="n">
         <v>46244</v>
       </c>
-      <c r="B4" s="4" t="n">
+      <c r="B4" s="2" t="n">
+        <v>46248</v>
+      </c>
+      <c r="C4" s="4" t="n">
         <v>2380.25</v>
       </c>
-      <c r="C4" s="4" t="n">
+      <c r="D4" s="4" t="n">
         <v>2344.55</v>
       </c>
-      <c r="D4" s="5" t="n">
+      <c r="E4" s="5" t="n">
         <v>67940689</v>
       </c>
-      <c r="E4" t="inlineStr"/>
+      <c r="F4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" s="2" t="n">
         <v>46251</v>
       </c>
-      <c r="B5" s="4" t="n">
+      <c r="B5" s="2" t="n">
+        <v>46255</v>
+      </c>
+      <c r="C5" s="4" t="n">
         <v>2436.27</v>
       </c>
-      <c r="C5" s="4" t="n">
+      <c r="D5" s="4" t="n">
         <v>2399.73</v>
       </c>
-      <c r="D5" s="5" t="n">
+      <c r="E5" s="5" t="n">
         <v>89707598</v>
       </c>
-      <c r="E5" t="inlineStr"/>
+      <c r="F5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" s="2" t="n">
         <v>46258</v>
       </c>
-      <c r="B6" s="4" t="n">
+      <c r="B6" s="2" t="n">
+        <v>46262</v>
+      </c>
+      <c r="C6" s="4" t="n">
         <v>2491.55</v>
       </c>
-      <c r="C6" s="4" t="n">
+      <c r="D6" s="4" t="n">
         <v>2454.18</v>
       </c>
-      <c r="D6" s="5" t="n">
+      <c r="E6" s="5" t="n">
         <v>6617569</v>
       </c>
-      <c r="E6" t="inlineStr"/>
+      <c r="F6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" s="2" t="n">
         <v>46265</v>
       </c>
-      <c r="B7" s="4" t="n">
+      <c r="B7" s="2" t="n">
+        <v>46265</v>
+      </c>
+      <c r="C7" s="4" t="n">
         <v>2501.12</v>
       </c>
-      <c r="C7" s="4" t="n">
+      <c r="D7" s="4" t="n">
         <v>2463.6</v>
       </c>
-      <c r="D7" s="5" t="n">
+      <c r="E7" s="5" t="n">
         <v>45992922</v>
       </c>
-      <c r="E7" t="inlineStr">
+      <c r="F7" t="inlineStr">
         <is>
           <t>Partial 未完整</t>
         </is>
@@ -1995,38 +2157,44 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E7"/>
+  <dimension ref="A1:F7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
-    <col width="16" customWidth="1" min="2" max="2"/>
-    <col width="22" customWidth="1" min="3" max="3"/>
-    <col width="16" customWidth="1" min="4" max="4"/>
-    <col width="20" customWidth="1" min="5" max="5"/>
+    <col width="15" customWidth="1" min="2" max="2"/>
+    <col width="16" customWidth="1" min="3" max="3"/>
+    <col width="24" customWidth="1" min="4" max="4"/>
+    <col width="16" customWidth="1" min="5" max="5"/>
+    <col width="22" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1" ht="32" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Date 日期</t>
+          <t>Period 期間</t>
         </is>
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
+          <t>Trade Date 取值日</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
           <t>Close 收盤價</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>Adj Close 調整後收盤價</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>Volume 成交量</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>Flag 註記</t>
         </is>
@@ -2036,16 +2204,19 @@
       <c r="A2" s="2" t="n">
         <v>46230</v>
       </c>
-      <c r="B2" s="4" t="n">
+      <c r="B2" s="2" t="n">
+        <v>46234</v>
+      </c>
+      <c r="C2" s="4" t="n">
         <v>149.91</v>
       </c>
-      <c r="C2" s="4" t="n">
+      <c r="D2" s="4" t="n">
         <v>147.66</v>
       </c>
-      <c r="D2" s="5" t="n">
+      <c r="E2" s="5" t="n">
         <v>77131377</v>
       </c>
-      <c r="E2" t="inlineStr">
+      <c r="F2" t="inlineStr">
         <is>
           <t>Prior period 前一期</t>
         </is>
@@ -2055,76 +2226,91 @@
       <c r="A3" s="2" t="n">
         <v>46237</v>
       </c>
-      <c r="B3" s="4" t="n">
+      <c r="B3" s="2" t="n">
+        <v>46241</v>
+      </c>
+      <c r="C3" s="4" t="n">
         <v>153.76</v>
       </c>
-      <c r="C3" s="4" t="n">
+      <c r="D3" s="4" t="n">
         <v>151.45</v>
       </c>
-      <c r="D3" s="5" t="n">
+      <c r="E3" s="5" t="n">
         <v>64498494</v>
       </c>
-      <c r="E3" t="inlineStr"/>
+      <c r="F3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" s="2" t="n">
         <v>46244</v>
       </c>
-      <c r="B4" s="4" t="n">
+      <c r="B4" s="2" t="n">
+        <v>46248</v>
+      </c>
+      <c r="C4" s="4" t="n">
         <v>153.67</v>
       </c>
-      <c r="C4" s="4" t="n">
+      <c r="D4" s="4" t="n">
         <v>151.36</v>
       </c>
-      <c r="D4" s="5" t="n">
+      <c r="E4" s="5" t="n">
         <v>80837457</v>
       </c>
-      <c r="E4" t="inlineStr"/>
+      <c r="F4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" s="2" t="n">
         <v>46251</v>
       </c>
-      <c r="B5" s="4" t="n">
+      <c r="B5" s="2" t="n">
+        <v>46255</v>
+      </c>
+      <c r="C5" s="4" t="n">
         <v>150.95</v>
       </c>
-      <c r="C5" s="4" t="n">
+      <c r="D5" s="4" t="n">
         <v>148.69</v>
       </c>
-      <c r="D5" s="5" t="n">
+      <c r="E5" s="5" t="n">
         <v>70707214</v>
       </c>
-      <c r="E5" t="inlineStr"/>
+      <c r="F5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" s="2" t="n">
         <v>46258</v>
       </c>
-      <c r="B6" s="4" t="n">
+      <c r="B6" s="2" t="n">
+        <v>46262</v>
+      </c>
+      <c r="C6" s="4" t="n">
         <v>151.09</v>
       </c>
-      <c r="C6" s="4" t="n">
+      <c r="D6" s="4" t="n">
         <v>148.82</v>
       </c>
-      <c r="D6" s="5" t="n">
+      <c r="E6" s="5" t="n">
         <v>84404159</v>
       </c>
-      <c r="E6" t="inlineStr"/>
+      <c r="F6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" s="2" t="n">
         <v>46265</v>
       </c>
-      <c r="B7" s="4" t="n">
+      <c r="B7" s="2" t="n">
+        <v>46265</v>
+      </c>
+      <c r="C7" s="4" t="n">
         <v>154.35</v>
       </c>
-      <c r="C7" s="4" t="n">
+      <c r="D7" s="4" t="n">
         <v>152.03</v>
       </c>
-      <c r="D7" s="5" t="n">
+      <c r="E7" s="5" t="n">
         <v>14633036</v>
       </c>
-      <c r="E7" t="inlineStr">
+      <c r="F7" t="inlineStr">
         <is>
           <t>Partial 未完整</t>
         </is>
@@ -2141,38 +2327,44 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E7"/>
+  <dimension ref="A1:F7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
-    <col width="16" customWidth="1" min="2" max="2"/>
-    <col width="22" customWidth="1" min="3" max="3"/>
-    <col width="16" customWidth="1" min="4" max="4"/>
-    <col width="20" customWidth="1" min="5" max="5"/>
+    <col width="15" customWidth="1" min="2" max="2"/>
+    <col width="16" customWidth="1" min="3" max="3"/>
+    <col width="24" customWidth="1" min="4" max="4"/>
+    <col width="16" customWidth="1" min="5" max="5"/>
+    <col width="22" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1" ht="32" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Date 日期</t>
+          <t>Period 期間</t>
         </is>
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
+          <t>Trade Date 取值日</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
           <t>Close 收盤價</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>Adj Close 調整後收盤價</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>Volume 成交量</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>Flag 註記</t>
         </is>
@@ -2182,16 +2374,19 @@
       <c r="A2" s="2" t="n">
         <v>46230</v>
       </c>
-      <c r="B2" s="4" t="n">
+      <c r="B2" s="2" t="n">
+        <v>46234</v>
+      </c>
+      <c r="C2" s="4" t="n">
         <v>230.19</v>
       </c>
-      <c r="C2" s="4" t="n">
+      <c r="D2" s="4" t="n">
         <v>226.74</v>
       </c>
-      <c r="D2" s="5" t="n">
+      <c r="E2" s="5" t="n">
         <v>73018730</v>
       </c>
-      <c r="E2" t="inlineStr">
+      <c r="F2" t="inlineStr">
         <is>
           <t>Prior period 前一期</t>
         </is>
@@ -2201,76 +2396,91 @@
       <c r="A3" s="2" t="n">
         <v>46237</v>
       </c>
-      <c r="B3" s="4" t="n">
+      <c r="B3" s="2" t="n">
+        <v>46241</v>
+      </c>
+      <c r="C3" s="4" t="n">
         <v>233.26</v>
       </c>
-      <c r="C3" s="4" t="n">
+      <c r="D3" s="4" t="n">
         <v>229.76</v>
       </c>
-      <c r="D3" s="5" t="n">
+      <c r="E3" s="5" t="n">
         <v>21139495</v>
       </c>
-      <c r="E3" t="inlineStr"/>
+      <c r="F3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" s="2" t="n">
         <v>46244</v>
       </c>
-      <c r="B4" s="4" t="n">
+      <c r="B4" s="2" t="n">
+        <v>46248</v>
+      </c>
+      <c r="C4" s="4" t="n">
         <v>232.05</v>
       </c>
-      <c r="C4" s="4" t="n">
+      <c r="D4" s="4" t="n">
         <v>228.57</v>
       </c>
-      <c r="D4" s="5" t="n">
+      <c r="E4" s="5" t="n">
         <v>52298696</v>
       </c>
-      <c r="E4" t="inlineStr"/>
+      <c r="F4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" s="2" t="n">
         <v>46251</v>
       </c>
-      <c r="B5" s="4" t="n">
+      <c r="B5" s="2" t="n">
+        <v>46255</v>
+      </c>
+      <c r="C5" s="4" t="n">
         <v>232.37</v>
       </c>
-      <c r="C5" s="4" t="n">
+      <c r="D5" s="4" t="n">
         <v>228.88</v>
       </c>
-      <c r="D5" s="5" t="n">
+      <c r="E5" s="5" t="n">
         <v>88356860</v>
       </c>
-      <c r="E5" t="inlineStr"/>
+      <c r="F5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" s="2" t="n">
         <v>46258</v>
       </c>
-      <c r="B6" s="4" t="n">
+      <c r="B6" s="2" t="n">
+        <v>46262</v>
+      </c>
+      <c r="C6" s="4" t="n">
         <v>237.63</v>
       </c>
-      <c r="C6" s="4" t="n">
+      <c r="D6" s="4" t="n">
         <v>234.07</v>
       </c>
-      <c r="D6" s="5" t="n">
+      <c r="E6" s="5" t="n">
         <v>82726197</v>
       </c>
-      <c r="E6" t="inlineStr"/>
+      <c r="F6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" s="2" t="n">
         <v>46265</v>
       </c>
-      <c r="B7" s="4" t="n">
+      <c r="B7" s="2" t="n">
+        <v>46265</v>
+      </c>
+      <c r="C7" s="4" t="n">
         <v>234.02</v>
       </c>
-      <c r="C7" s="4" t="n">
+      <c r="D7" s="4" t="n">
         <v>230.51</v>
       </c>
-      <c r="D7" s="5" t="n">
+      <c r="E7" s="5" t="n">
         <v>2223590</v>
       </c>
-      <c r="E7" t="inlineStr">
+      <c r="F7" t="inlineStr">
         <is>
           <t>Partial 未完整</t>
         </is>
@@ -2287,38 +2497,44 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E7"/>
+  <dimension ref="A1:F7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
-    <col width="16" customWidth="1" min="2" max="2"/>
-    <col width="22" customWidth="1" min="3" max="3"/>
-    <col width="16" customWidth="1" min="4" max="4"/>
-    <col width="20" customWidth="1" min="5" max="5"/>
+    <col width="15" customWidth="1" min="2" max="2"/>
+    <col width="16" customWidth="1" min="3" max="3"/>
+    <col width="24" customWidth="1" min="4" max="4"/>
+    <col width="16" customWidth="1" min="5" max="5"/>
+    <col width="22" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1" ht="32" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Date 日期</t>
+          <t>Period 期間</t>
         </is>
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
+          <t>Trade Date 取值日</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
           <t>Close 收盤價</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>Adj Close 調整後收盤價</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>Volume 成交量</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>Flag 註記</t>
         </is>
@@ -2328,16 +2544,19 @@
       <c r="A2" s="2" t="n">
         <v>46230</v>
       </c>
-      <c r="B2" s="4" t="n">
+      <c r="B2" s="2" t="n">
+        <v>46234</v>
+      </c>
+      <c r="C2" s="4" t="n">
         <v>286.18</v>
       </c>
-      <c r="C2" s="4" t="n">
+      <c r="D2" s="4" t="n">
         <v>281.89</v>
       </c>
-      <c r="D2" s="5" t="n">
+      <c r="E2" s="5" t="n">
         <v>26927476</v>
       </c>
-      <c r="E2" t="inlineStr">
+      <c r="F2" t="inlineStr">
         <is>
           <t>Prior period 前一期</t>
         </is>
@@ -2347,76 +2566,91 @@
       <c r="A3" s="2" t="n">
         <v>46237</v>
       </c>
-      <c r="B3" s="4" t="n">
+      <c r="B3" s="2" t="n">
+        <v>46241</v>
+      </c>
+      <c r="C3" s="4" t="n">
         <v>289.73</v>
       </c>
-      <c r="C3" s="4" t="n">
+      <c r="D3" s="4" t="n">
         <v>285.38</v>
       </c>
-      <c r="D3" s="5" t="n">
+      <c r="E3" s="5" t="n">
         <v>21751469</v>
       </c>
-      <c r="E3" t="inlineStr"/>
+      <c r="F3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" s="2" t="n">
         <v>46244</v>
       </c>
-      <c r="B4" s="4" t="n">
+      <c r="B4" s="2" t="n">
+        <v>46248</v>
+      </c>
+      <c r="C4" s="4" t="n">
         <v>297.4</v>
       </c>
-      <c r="C4" s="4" t="n">
+      <c r="D4" s="4" t="n">
         <v>292.94</v>
       </c>
-      <c r="D4" s="5" t="n">
+      <c r="E4" s="5" t="n">
         <v>88027814</v>
       </c>
-      <c r="E4" t="inlineStr"/>
+      <c r="F4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" s="2" t="n">
         <v>46251</v>
       </c>
-      <c r="B5" s="4" t="n">
+      <c r="B5" s="2" t="n">
+        <v>46255</v>
+      </c>
+      <c r="C5" s="4" t="n">
         <v>302.67</v>
       </c>
-      <c r="C5" s="4" t="n">
+      <c r="D5" s="4" t="n">
         <v>298.13</v>
       </c>
-      <c r="D5" s="5" t="n">
+      <c r="E5" s="5" t="n">
         <v>19476896</v>
       </c>
-      <c r="E5" t="inlineStr"/>
+      <c r="F5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" s="2" t="n">
         <v>46258</v>
       </c>
-      <c r="B6" s="4" t="n">
+      <c r="B6" s="2" t="n">
+        <v>46262</v>
+      </c>
+      <c r="C6" s="4" t="n">
         <v>294.98</v>
       </c>
-      <c r="C6" s="4" t="n">
+      <c r="D6" s="4" t="n">
         <v>290.56</v>
       </c>
-      <c r="D6" s="5" t="n">
+      <c r="E6" s="5" t="n">
         <v>30710182</v>
       </c>
-      <c r="E6" t="inlineStr"/>
+      <c r="F6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" s="2" t="n">
         <v>46265</v>
       </c>
-      <c r="B7" s="4" t="n">
+      <c r="B7" s="2" t="n">
+        <v>46265</v>
+      </c>
+      <c r="C7" s="4" t="n">
         <v>300.41</v>
       </c>
-      <c r="C7" s="4" t="n">
+      <c r="D7" s="4" t="n">
         <v>295.9</v>
       </c>
-      <c r="D7" s="5" t="n">
+      <c r="E7" s="5" t="n">
         <v>6023039</v>
       </c>
-      <c r="E7" t="inlineStr">
+      <c r="F7" t="inlineStr">
         <is>
           <t>Partial 未完整</t>
         </is>
@@ -2433,38 +2667,44 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E7"/>
+  <dimension ref="A1:F7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
-    <col width="16" customWidth="1" min="2" max="2"/>
-    <col width="22" customWidth="1" min="3" max="3"/>
-    <col width="16" customWidth="1" min="4" max="4"/>
-    <col width="20" customWidth="1" min="5" max="5"/>
+    <col width="15" customWidth="1" min="2" max="2"/>
+    <col width="16" customWidth="1" min="3" max="3"/>
+    <col width="24" customWidth="1" min="4" max="4"/>
+    <col width="16" customWidth="1" min="5" max="5"/>
+    <col width="22" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1" ht="32" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Date 日期</t>
+          <t>Period 期間</t>
         </is>
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
+          <t>Trade Date 取值日</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
           <t>Close 收盤價</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>Adj Close 調整後收盤價</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>Volume 成交量</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>Flag 註記</t>
         </is>
@@ -2474,16 +2714,19 @@
       <c r="A2" s="2" t="n">
         <v>46230</v>
       </c>
-      <c r="B2" s="4" t="n">
+      <c r="B2" s="2" t="n">
+        <v>46234</v>
+      </c>
+      <c r="C2" s="4" t="n">
         <v>117.23</v>
       </c>
-      <c r="C2" s="4" t="n">
+      <c r="D2" s="4" t="n">
         <v>115.47</v>
       </c>
-      <c r="D2" s="5" t="n">
+      <c r="E2" s="5" t="n">
         <v>89515598</v>
       </c>
-      <c r="E2" t="inlineStr">
+      <c r="F2" t="inlineStr">
         <is>
           <t>Prior period 前一期</t>
         </is>
@@ -2493,76 +2736,91 @@
       <c r="A3" s="2" t="n">
         <v>46237</v>
       </c>
-      <c r="B3" s="4" t="n">
+      <c r="B3" s="2" t="n">
+        <v>46241</v>
+      </c>
+      <c r="C3" s="4" t="n">
         <v>117.73</v>
       </c>
-      <c r="C3" s="4" t="n">
+      <c r="D3" s="4" t="n">
         <v>115.96</v>
       </c>
-      <c r="D3" s="5" t="n">
+      <c r="E3" s="5" t="n">
         <v>35143088</v>
       </c>
-      <c r="E3" t="inlineStr"/>
+      <c r="F3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" s="2" t="n">
         <v>46244</v>
       </c>
-      <c r="B4" s="4" t="n">
+      <c r="B4" s="2" t="n">
+        <v>46248</v>
+      </c>
+      <c r="C4" s="4" t="n">
         <v>116.28</v>
       </c>
-      <c r="C4" s="4" t="n">
+      <c r="D4" s="4" t="n">
         <v>114.54</v>
       </c>
-      <c r="D4" s="5" t="n">
+      <c r="E4" s="5" t="n">
         <v>36329608</v>
       </c>
-      <c r="E4" t="inlineStr"/>
+      <c r="F4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" s="2" t="n">
         <v>46251</v>
       </c>
-      <c r="B5" s="4" t="n">
+      <c r="B5" s="2" t="n">
+        <v>46255</v>
+      </c>
+      <c r="C5" s="4" t="n">
         <v>114.99</v>
       </c>
-      <c r="C5" s="4" t="n">
+      <c r="D5" s="4" t="n">
         <v>113.27</v>
       </c>
-      <c r="D5" s="5" t="n">
+      <c r="E5" s="5" t="n">
         <v>11747679</v>
       </c>
-      <c r="E5" t="inlineStr"/>
+      <c r="F5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" s="2" t="n">
         <v>46258</v>
       </c>
-      <c r="B6" s="4" t="n">
+      <c r="B6" s="2" t="n">
+        <v>46262</v>
+      </c>
+      <c r="C6" s="4" t="n">
         <v>116.46</v>
       </c>
-      <c r="C6" s="4" t="n">
+      <c r="D6" s="4" t="n">
         <v>114.71</v>
       </c>
-      <c r="D6" s="5" t="n">
+      <c r="E6" s="5" t="n">
         <v>42666357</v>
       </c>
-      <c r="E6" t="inlineStr"/>
+      <c r="F6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" s="2" t="n">
         <v>46265</v>
       </c>
-      <c r="B7" s="4" t="n">
+      <c r="B7" s="2" t="n">
+        <v>46265</v>
+      </c>
+      <c r="C7" s="4" t="n">
         <v>116.5</v>
       </c>
-      <c r="C7" s="4" t="n">
+      <c r="D7" s="4" t="n">
         <v>114.75</v>
       </c>
-      <c r="D7" s="5" t="n">
+      <c r="E7" s="5" t="n">
         <v>55240635</v>
       </c>
-      <c r="E7" t="inlineStr">
+      <c r="F7" t="inlineStr">
         <is>
           <t>Partial 未完整</t>
         </is>
@@ -2604,7 +2862,7 @@
     <row r="1" ht="32" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Date 日期</t>
+          <t>Period 期間</t>
         </is>
       </c>
       <c r="B1" s="1" t="inlineStr">
@@ -3036,7 +3294,7 @@
     <row r="1" ht="32" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Date 日期</t>
+          <t>Period 期間</t>
         </is>
       </c>
       <c r="B1" s="1" t="inlineStr">
@@ -3443,38 +3701,44 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E7"/>
+  <dimension ref="A1:F7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
-    <col width="16" customWidth="1" min="2" max="2"/>
-    <col width="22" customWidth="1" min="3" max="3"/>
-    <col width="16" customWidth="1" min="4" max="4"/>
-    <col width="20" customWidth="1" min="5" max="5"/>
+    <col width="15" customWidth="1" min="2" max="2"/>
+    <col width="16" customWidth="1" min="3" max="3"/>
+    <col width="24" customWidth="1" min="4" max="4"/>
+    <col width="16" customWidth="1" min="5" max="5"/>
+    <col width="22" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1" ht="32" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Date 日期</t>
+          <t>Period 期間</t>
         </is>
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
+          <t>Trade Date 取值日</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
           <t>Close 收盤價</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>Adj Close 調整後收盤價</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>Volume 成交量</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>Flag 註記</t>
         </is>
@@ -3484,16 +3748,19 @@
       <c r="A2" s="2" t="n">
         <v>46230</v>
       </c>
-      <c r="B2" s="4" t="n">
+      <c r="B2" s="2" t="n">
+        <v>46234</v>
+      </c>
+      <c r="C2" s="4" t="n">
         <v>44070.16</v>
       </c>
-      <c r="C2" s="4" t="n">
+      <c r="D2" s="4" t="n">
         <v>43409.11</v>
       </c>
-      <c r="D2" s="5" t="n">
+      <c r="E2" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="E2" t="inlineStr">
+      <c r="F2" t="inlineStr">
         <is>
           <t>Prior period 前一期</t>
         </is>
@@ -3503,76 +3770,91 @@
       <c r="A3" s="2" t="n">
         <v>46237</v>
       </c>
-      <c r="B3" s="4" t="n">
+      <c r="B3" s="2" t="n">
+        <v>46241</v>
+      </c>
+      <c r="C3" s="4" t="n">
         <v>44919.26</v>
       </c>
-      <c r="C3" s="4" t="n">
+      <c r="D3" s="4" t="n">
         <v>44245.47</v>
       </c>
-      <c r="D3" s="5" t="n">
+      <c r="E3" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="E3" t="inlineStr"/>
+      <c r="F3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" s="2" t="n">
         <v>46244</v>
       </c>
-      <c r="B4" s="4" t="n">
+      <c r="B4" s="2" t="n">
+        <v>46248</v>
+      </c>
+      <c r="C4" s="4" t="n">
         <v>44799.65</v>
       </c>
-      <c r="C4" s="4" t="n">
+      <c r="D4" s="4" t="n">
         <v>44127.66</v>
       </c>
-      <c r="D4" s="5" t="n">
+      <c r="E4" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="E4" t="inlineStr"/>
+      <c r="F4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" s="2" t="n">
-        <v>46252</v>
-      </c>
-      <c r="B5" s="4" t="n">
+        <v>46251</v>
+      </c>
+      <c r="B5" s="2" t="n">
+        <v>46254</v>
+      </c>
+      <c r="C5" s="4" t="n">
         <v>44209.62</v>
       </c>
-      <c r="C5" s="4" t="n">
+      <c r="D5" s="4" t="n">
         <v>43546.48</v>
       </c>
-      <c r="D5" s="5" t="n">
+      <c r="E5" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="E5" t="inlineStr"/>
+      <c r="F5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" s="2" t="n">
         <v>46258</v>
       </c>
-      <c r="B6" s="4" t="n">
+      <c r="B6" s="2" t="n">
+        <v>46262</v>
+      </c>
+      <c r="C6" s="4" t="n">
         <v>44352.54</v>
       </c>
-      <c r="C6" s="4" t="n">
+      <c r="D6" s="4" t="n">
         <v>43687.25</v>
       </c>
-      <c r="D6" s="5" t="n">
+      <c r="E6" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="E6" t="inlineStr"/>
+      <c r="F6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" s="2" t="n">
         <v>46265</v>
       </c>
-      <c r="B7" s="4" t="n">
+      <c r="B7" s="2" t="n">
+        <v>46265</v>
+      </c>
+      <c r="C7" s="4" t="n">
         <v>44189.36</v>
       </c>
-      <c r="C7" s="4" t="n">
+      <c r="D7" s="4" t="n">
         <v>43526.52</v>
       </c>
-      <c r="D7" s="5" t="n">
+      <c r="E7" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="E7" t="inlineStr">
+      <c r="F7" t="inlineStr">
         <is>
           <t>Partial 未完整</t>
         </is>
@@ -3589,38 +3871,44 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E6"/>
+  <dimension ref="A1:F7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
-    <col width="16" customWidth="1" min="2" max="2"/>
-    <col width="22" customWidth="1" min="3" max="3"/>
-    <col width="16" customWidth="1" min="4" max="4"/>
-    <col width="20" customWidth="1" min="5" max="5"/>
+    <col width="15" customWidth="1" min="2" max="2"/>
+    <col width="16" customWidth="1" min="3" max="3"/>
+    <col width="24" customWidth="1" min="4" max="4"/>
+    <col width="16" customWidth="1" min="5" max="5"/>
+    <col width="22" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1" ht="32" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Date 日期</t>
+          <t>Period 期間</t>
         </is>
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
+          <t>Trade Date 取值日</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
           <t>Close 收盤價</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>Adj Close 調整後收盤價</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>Volume 成交量</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>Flag 註記</t>
         </is>
@@ -3630,16 +3918,19 @@
       <c r="A2" s="2" t="n">
         <v>46230</v>
       </c>
-      <c r="B2" s="4" t="n">
+      <c r="B2" s="2" t="n">
+        <v>46234</v>
+      </c>
+      <c r="C2" s="4" t="n">
         <v>39149.35</v>
       </c>
-      <c r="C2" s="4" t="n">
+      <c r="D2" s="4" t="n">
         <v>38562.11</v>
       </c>
-      <c r="D2" s="5" t="n">
+      <c r="E2" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="E2" t="inlineStr">
+      <c r="F2" t="inlineStr">
         <is>
           <t>Prior period 前一期</t>
         </is>
@@ -3649,61 +3940,87 @@
       <c r="A3" s="2" t="n">
         <v>46237</v>
       </c>
-      <c r="B3" s="4" t="n">
+      <c r="B3" s="2" t="n">
+        <v>46241</v>
+      </c>
+      <c r="C3" s="4" t="n">
         <v>40131.34</v>
       </c>
-      <c r="C3" s="4" t="n">
+      <c r="D3" s="4" t="n">
         <v>39529.37</v>
       </c>
-      <c r="D3" s="5" t="n">
+      <c r="E3" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="E3" t="inlineStr"/>
+      <c r="F3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" s="2" t="n">
-        <v>46251</v>
-      </c>
-      <c r="B4" s="4" t="n">
-        <v>40370.57</v>
-      </c>
-      <c r="C4" s="4" t="n">
-        <v>39765.01</v>
-      </c>
-      <c r="D4" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="E4" t="inlineStr"/>
+        <v>46244</v>
+      </c>
+      <c r="B4" s="2" t="n"/>
+      <c r="C4" s="4" t="n"/>
+      <c r="D4" s="4" t="n"/>
+      <c r="E4" s="5" t="n"/>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>No trading 休市</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="n">
-        <v>46258</v>
-      </c>
-      <c r="B5" s="4" t="n">
-        <v>40459.52</v>
+        <v>46251</v>
+      </c>
+      <c r="B5" s="2" t="n">
+        <v>46255</v>
       </c>
       <c r="C5" s="4" t="n">
-        <v>39852.63</v>
-      </c>
-      <c r="D5" s="5" t="n">
+        <v>40370.57</v>
+      </c>
+      <c r="D5" s="4" t="n">
+        <v>39765.01</v>
+      </c>
+      <c r="E5" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="E5" t="inlineStr"/>
+      <c r="F5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" s="2" t="n">
+        <v>46258</v>
+      </c>
+      <c r="B6" s="2" t="n">
+        <v>46262</v>
+      </c>
+      <c r="C6" s="4" t="n">
+        <v>40459.52</v>
+      </c>
+      <c r="D6" s="4" t="n">
+        <v>39852.63</v>
+      </c>
+      <c r="E6" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="F6" t="inlineStr"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="n">
         <v>46265</v>
       </c>
-      <c r="B6" s="4" t="n">
+      <c r="B7" s="2" t="n">
+        <v>46265</v>
+      </c>
+      <c r="C7" s="4" t="n">
         <v>40427.83</v>
       </c>
-      <c r="C6" s="4" t="n">
+      <c r="D7" s="4" t="n">
         <v>39821.41</v>
       </c>
-      <c r="D6" s="5" t="n">
+      <c r="E7" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="E6" t="inlineStr">
+      <c r="F7" t="inlineStr">
         <is>
           <t>Partial 未完整</t>
         </is>
@@ -3720,38 +4037,44 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E7"/>
+  <dimension ref="A1:F7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
-    <col width="16" customWidth="1" min="2" max="2"/>
-    <col width="22" customWidth="1" min="3" max="3"/>
-    <col width="16" customWidth="1" min="4" max="4"/>
-    <col width="20" customWidth="1" min="5" max="5"/>
+    <col width="15" customWidth="1" min="2" max="2"/>
+    <col width="16" customWidth="1" min="3" max="3"/>
+    <col width="24" customWidth="1" min="4" max="4"/>
+    <col width="16" customWidth="1" min="5" max="5"/>
+    <col width="22" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1" ht="32" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Date 日期</t>
+          <t>Period 期間</t>
         </is>
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
+          <t>Trade Date 取值日</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
           <t>Close 收盤價</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>Adj Close 調整後收盤價</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>Volume 成交量</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>Flag 註記</t>
         </is>
@@ -3761,16 +4084,19 @@
       <c r="A2" s="2" t="n">
         <v>46230</v>
       </c>
-      <c r="B2" s="4" t="n">
+      <c r="B2" s="2" t="n">
+        <v>46234</v>
+      </c>
+      <c r="C2" s="4" t="n">
         <v>768.95</v>
       </c>
-      <c r="C2" s="4" t="n">
+      <c r="D2" s="4" t="n">
         <v>757.42</v>
       </c>
-      <c r="D2" s="5" t="n">
+      <c r="E2" s="5" t="n">
         <v>9590196</v>
       </c>
-      <c r="E2" t="inlineStr">
+      <c r="F2" t="inlineStr">
         <is>
           <t>Prior period 前一期</t>
         </is>
@@ -3780,76 +4106,91 @@
       <c r="A3" s="2" t="n">
         <v>46237</v>
       </c>
-      <c r="B3" s="4" t="n">
+      <c r="B3" s="2" t="n">
+        <v>46241</v>
+      </c>
+      <c r="C3" s="4" t="n">
         <v>750.46</v>
       </c>
-      <c r="C3" s="4" t="n">
+      <c r="D3" s="4" t="n">
         <v>739.2</v>
       </c>
-      <c r="D3" s="5" t="n">
+      <c r="E3" s="5" t="n">
         <v>50460313</v>
       </c>
-      <c r="E3" t="inlineStr"/>
+      <c r="F3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" s="2" t="n">
         <v>46244</v>
       </c>
-      <c r="B4" s="4" t="n">
+      <c r="B4" s="2" t="n">
+        <v>46248</v>
+      </c>
+      <c r="C4" s="4" t="n">
         <v>768.7</v>
       </c>
-      <c r="C4" s="4" t="n">
+      <c r="D4" s="4" t="n">
         <v>757.17</v>
       </c>
-      <c r="D4" s="5" t="n">
+      <c r="E4" s="5" t="n">
         <v>43357375</v>
       </c>
-      <c r="E4" t="inlineStr"/>
+      <c r="F4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" s="2" t="n">
         <v>46251</v>
       </c>
-      <c r="B5" s="4" t="n">
+      <c r="B5" s="2" t="n">
+        <v>46255</v>
+      </c>
+      <c r="C5" s="4" t="n">
         <v>758.21</v>
       </c>
-      <c r="C5" s="4" t="n">
+      <c r="D5" s="4" t="n">
         <v>746.84</v>
       </c>
-      <c r="D5" s="5" t="n">
+      <c r="E5" s="5" t="n">
         <v>30483526</v>
       </c>
-      <c r="E5" t="inlineStr"/>
+      <c r="F5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" s="2" t="n">
         <v>46258</v>
       </c>
-      <c r="B6" s="4" t="n">
+      <c r="B6" s="2" t="n">
+        <v>46262</v>
+      </c>
+      <c r="C6" s="4" t="n">
         <v>765.37</v>
       </c>
-      <c r="C6" s="4" t="n">
+      <c r="D6" s="4" t="n">
         <v>753.89</v>
       </c>
-      <c r="D6" s="5" t="n">
+      <c r="E6" s="5" t="n">
         <v>80007882</v>
       </c>
-      <c r="E6" t="inlineStr"/>
+      <c r="F6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" s="2" t="n">
         <v>46265</v>
       </c>
-      <c r="B7" s="4" t="n">
+      <c r="B7" s="2" t="n">
+        <v>46265</v>
+      </c>
+      <c r="C7" s="4" t="n">
         <v>776.3</v>
       </c>
-      <c r="C7" s="4" t="n">
+      <c r="D7" s="4" t="n">
         <v>764.66</v>
       </c>
-      <c r="D7" s="5" t="n">
+      <c r="E7" s="5" t="n">
         <v>59803500</v>
       </c>
-      <c r="E7" t="inlineStr">
+      <c r="F7" t="inlineStr">
         <is>
           <t>Partial 未完整</t>
         </is>
@@ -3866,38 +4207,44 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E7"/>
+  <dimension ref="A1:F7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
-    <col width="16" customWidth="1" min="2" max="2"/>
-    <col width="22" customWidth="1" min="3" max="3"/>
-    <col width="16" customWidth="1" min="4" max="4"/>
-    <col width="20" customWidth="1" min="5" max="5"/>
+    <col width="15" customWidth="1" min="2" max="2"/>
+    <col width="16" customWidth="1" min="3" max="3"/>
+    <col width="24" customWidth="1" min="4" max="4"/>
+    <col width="16" customWidth="1" min="5" max="5"/>
+    <col width="22" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1" ht="32" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Date 日期</t>
+          <t>Period 期間</t>
         </is>
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
+          <t>Trade Date 取值日</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
           <t>Close 收盤價</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>Adj Close 調整後收盤價</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>Volume 成交量</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>Flag 註記</t>
         </is>
@@ -3907,16 +4254,19 @@
       <c r="A2" s="2" t="n">
         <v>46230</v>
       </c>
-      <c r="B2" s="4" t="n">
+      <c r="B2" s="2" t="n">
+        <v>46234</v>
+      </c>
+      <c r="C2" s="4" t="n">
         <v>68.98</v>
       </c>
-      <c r="C2" s="4" t="n">
+      <c r="D2" s="4" t="n">
         <v>67.95</v>
       </c>
-      <c r="D2" s="5" t="n">
+      <c r="E2" s="5" t="n">
         <v>75045210</v>
       </c>
-      <c r="E2" t="inlineStr">
+      <c r="F2" t="inlineStr">
         <is>
           <t>Prior period 前一期</t>
         </is>
@@ -3926,76 +4276,91 @@
       <c r="A3" s="2" t="n">
         <v>46237</v>
       </c>
-      <c r="B3" s="4" t="n">
+      <c r="B3" s="2" t="n">
+        <v>46241</v>
+      </c>
+      <c r="C3" s="4" t="n">
         <v>67.5</v>
       </c>
-      <c r="C3" s="4" t="n">
+      <c r="D3" s="4" t="n">
         <v>66.48999999999999</v>
       </c>
-      <c r="D3" s="5" t="n">
+      <c r="E3" s="5" t="n">
         <v>83056775</v>
       </c>
-      <c r="E3" t="inlineStr"/>
+      <c r="F3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" s="2" t="n">
         <v>46244</v>
       </c>
-      <c r="B4" s="4" t="n">
+      <c r="B4" s="2" t="n">
+        <v>46248</v>
+      </c>
+      <c r="C4" s="4" t="n">
         <v>67.55</v>
       </c>
-      <c r="C4" s="4" t="n">
+      <c r="D4" s="4" t="n">
         <v>66.54000000000001</v>
       </c>
-      <c r="D4" s="5" t="n">
+      <c r="E4" s="5" t="n">
         <v>79960647</v>
       </c>
-      <c r="E4" t="inlineStr"/>
+      <c r="F4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" s="2" t="n">
         <v>46251</v>
       </c>
-      <c r="B5" s="4" t="n">
+      <c r="B5" s="2" t="n">
+        <v>46255</v>
+      </c>
+      <c r="C5" s="4" t="n">
         <v>65.81</v>
       </c>
-      <c r="C5" s="4" t="n">
+      <c r="D5" s="4" t="n">
         <v>64.81999999999999</v>
       </c>
-      <c r="D5" s="5" t="n">
+      <c r="E5" s="5" t="n">
         <v>3767377</v>
       </c>
-      <c r="E5" t="inlineStr"/>
+      <c r="F5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" s="2" t="n">
         <v>46258</v>
       </c>
-      <c r="B6" s="4" t="n">
+      <c r="B6" s="2" t="n">
+        <v>46262</v>
+      </c>
+      <c r="C6" s="4" t="n">
         <v>67.73</v>
       </c>
-      <c r="C6" s="4" t="n">
+      <c r="D6" s="4" t="n">
         <v>66.70999999999999</v>
       </c>
-      <c r="D6" s="5" t="n">
+      <c r="E6" s="5" t="n">
         <v>64979298</v>
       </c>
-      <c r="E6" t="inlineStr"/>
+      <c r="F6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" s="2" t="n">
         <v>46265</v>
       </c>
-      <c r="B7" s="4" t="n">
+      <c r="B7" s="2" t="n">
+        <v>46265</v>
+      </c>
+      <c r="C7" s="4" t="n">
         <v>66.84</v>
       </c>
-      <c r="C7" s="4" t="n">
+      <c r="D7" s="4" t="n">
         <v>65.84</v>
       </c>
-      <c r="D7" s="5" t="n">
+      <c r="E7" s="5" t="n">
         <v>33451369</v>
       </c>
-      <c r="E7" t="inlineStr">
+      <c r="F7" t="inlineStr">
         <is>
           <t>Partial 未完整</t>
         </is>
@@ -4012,38 +4377,44 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E7"/>
+  <dimension ref="A1:F7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
-    <col width="16" customWidth="1" min="2" max="2"/>
-    <col width="22" customWidth="1" min="3" max="3"/>
-    <col width="16" customWidth="1" min="4" max="4"/>
-    <col width="20" customWidth="1" min="5" max="5"/>
+    <col width="15" customWidth="1" min="2" max="2"/>
+    <col width="16" customWidth="1" min="3" max="3"/>
+    <col width="24" customWidth="1" min="4" max="4"/>
+    <col width="16" customWidth="1" min="5" max="5"/>
+    <col width="22" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1" ht="32" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Date 日期</t>
+          <t>Period 期間</t>
         </is>
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
+          <t>Trade Date 取值日</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
           <t>Close 收盤價</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>Adj Close 調整後收盤價</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>Volume 成交量</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>Flag 註記</t>
         </is>
@@ -4053,16 +4424,19 @@
       <c r="A2" s="2" t="n">
         <v>46230</v>
       </c>
-      <c r="B2" s="4" t="n">
+      <c r="B2" s="2" t="n">
+        <v>46234</v>
+      </c>
+      <c r="C2" s="4" t="n">
         <v>54.19</v>
       </c>
-      <c r="C2" s="4" t="n">
+      <c r="D2" s="4" t="n">
         <v>53.38</v>
       </c>
-      <c r="D2" s="5" t="n">
+      <c r="E2" s="5" t="n">
         <v>15846710</v>
       </c>
-      <c r="E2" t="inlineStr">
+      <c r="F2" t="inlineStr">
         <is>
           <t>Prior period 前一期</t>
         </is>
@@ -4072,76 +4446,91 @@
       <c r="A3" s="2" t="n">
         <v>46237</v>
       </c>
-      <c r="B3" s="4" t="n">
+      <c r="B3" s="2" t="n">
+        <v>46241</v>
+      </c>
+      <c r="C3" s="4" t="n">
         <v>55.11</v>
       </c>
-      <c r="C3" s="4" t="n">
+      <c r="D3" s="4" t="n">
         <v>54.28</v>
       </c>
-      <c r="D3" s="5" t="n">
+      <c r="E3" s="5" t="n">
         <v>66273970</v>
       </c>
-      <c r="E3" t="inlineStr"/>
+      <c r="F3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" s="2" t="n">
         <v>46244</v>
       </c>
-      <c r="B4" s="4" t="n">
+      <c r="B4" s="2" t="n">
+        <v>46248</v>
+      </c>
+      <c r="C4" s="4" t="n">
         <v>54.01</v>
       </c>
-      <c r="C4" s="4" t="n">
+      <c r="D4" s="4" t="n">
         <v>53.2</v>
       </c>
-      <c r="D4" s="5" t="n">
+      <c r="E4" s="5" t="n">
         <v>10927505</v>
       </c>
-      <c r="E4" t="inlineStr"/>
+      <c r="F4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" s="2" t="n">
         <v>46251</v>
       </c>
-      <c r="B5" s="4" t="n">
+      <c r="B5" s="2" t="n">
+        <v>46255</v>
+      </c>
+      <c r="C5" s="4" t="n">
         <v>52.46</v>
       </c>
-      <c r="C5" s="4" t="n">
+      <c r="D5" s="4" t="n">
         <v>51.67</v>
       </c>
-      <c r="D5" s="5" t="n">
+      <c r="E5" s="5" t="n">
         <v>75739467</v>
       </c>
-      <c r="E5" t="inlineStr"/>
+      <c r="F5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" s="2" t="n">
         <v>46258</v>
       </c>
-      <c r="B6" s="4" t="n">
+      <c r="B6" s="2" t="n">
+        <v>46262</v>
+      </c>
+      <c r="C6" s="4" t="n">
         <v>54.02</v>
       </c>
-      <c r="C6" s="4" t="n">
+      <c r="D6" s="4" t="n">
         <v>53.21</v>
       </c>
-      <c r="D6" s="5" t="n">
+      <c r="E6" s="5" t="n">
         <v>9898318</v>
       </c>
-      <c r="E6" t="inlineStr"/>
+      <c r="F6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" s="2" t="n">
         <v>46265</v>
       </c>
-      <c r="B7" s="4" t="n">
+      <c r="B7" s="2" t="n">
+        <v>46265</v>
+      </c>
+      <c r="C7" s="4" t="n">
         <v>53.17</v>
       </c>
-      <c r="C7" s="4" t="n">
+      <c r="D7" s="4" t="n">
         <v>52.37</v>
       </c>
-      <c r="D7" s="5" t="n">
+      <c r="E7" s="5" t="n">
         <v>74031971</v>
       </c>
-      <c r="E7" t="inlineStr">
+      <c r="F7" t="inlineStr">
         <is>
           <t>Partial 未完整</t>
         </is>
@@ -4158,38 +4547,44 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E7"/>
+  <dimension ref="A1:F7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
-    <col width="16" customWidth="1" min="2" max="2"/>
-    <col width="22" customWidth="1" min="3" max="3"/>
-    <col width="16" customWidth="1" min="4" max="4"/>
-    <col width="20" customWidth="1" min="5" max="5"/>
+    <col width="15" customWidth="1" min="2" max="2"/>
+    <col width="16" customWidth="1" min="3" max="3"/>
+    <col width="24" customWidth="1" min="4" max="4"/>
+    <col width="16" customWidth="1" min="5" max="5"/>
+    <col width="22" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1" ht="32" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Date 日期</t>
+          <t>Period 期間</t>
         </is>
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
+          <t>Trade Date 取值日</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
           <t>Close 收盤價</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>Adj Close 調整後收盤價</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>Volume 成交量</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>Flag 註記</t>
         </is>
@@ -4199,16 +4594,19 @@
       <c r="A2" s="2" t="n">
         <v>46230</v>
       </c>
-      <c r="B2" s="4" t="n">
+      <c r="B2" s="2" t="n">
+        <v>46234</v>
+      </c>
+      <c r="C2" s="4" t="n">
         <v>111.15</v>
       </c>
-      <c r="C2" s="4" t="n">
+      <c r="D2" s="4" t="n">
         <v>109.48</v>
       </c>
-      <c r="D2" s="5" t="n">
+      <c r="E2" s="5" t="n">
         <v>50121821</v>
       </c>
-      <c r="E2" t="inlineStr">
+      <c r="F2" t="inlineStr">
         <is>
           <t>Prior period 前一期</t>
         </is>
@@ -4218,76 +4616,91 @@
       <c r="A3" s="2" t="n">
         <v>46237</v>
       </c>
-      <c r="B3" s="4" t="n">
+      <c r="B3" s="2" t="n">
+        <v>46241</v>
+      </c>
+      <c r="C3" s="4" t="n">
         <v>113.56</v>
       </c>
-      <c r="C3" s="4" t="n">
+      <c r="D3" s="4" t="n">
         <v>111.86</v>
       </c>
-      <c r="D3" s="5" t="n">
+      <c r="E3" s="5" t="n">
         <v>89514212</v>
       </c>
-      <c r="E3" t="inlineStr"/>
+      <c r="F3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" s="2" t="n">
         <v>46244</v>
       </c>
-      <c r="B4" s="4" t="n">
+      <c r="B4" s="2" t="n">
+        <v>46248</v>
+      </c>
+      <c r="C4" s="4" t="n">
         <v>116.97</v>
       </c>
-      <c r="C4" s="4" t="n">
+      <c r="D4" s="4" t="n">
         <v>115.22</v>
       </c>
-      <c r="D4" s="5" t="n">
+      <c r="E4" s="5" t="n">
         <v>5893015</v>
       </c>
-      <c r="E4" t="inlineStr"/>
+      <c r="F4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" s="2" t="n">
         <v>46251</v>
       </c>
-      <c r="B5" s="4" t="n">
+      <c r="B5" s="2" t="n">
+        <v>46255</v>
+      </c>
+      <c r="C5" s="4" t="n">
         <v>119.85</v>
       </c>
-      <c r="C5" s="4" t="n">
+      <c r="D5" s="4" t="n">
         <v>118.05</v>
       </c>
-      <c r="D5" s="5" t="n">
+      <c r="E5" s="5" t="n">
         <v>35427281</v>
       </c>
-      <c r="E5" t="inlineStr"/>
+      <c r="F5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" s="2" t="n">
         <v>46258</v>
       </c>
-      <c r="B6" s="4" t="n">
+      <c r="B6" s="2" t="n">
+        <v>46262</v>
+      </c>
+      <c r="C6" s="4" t="n">
         <v>121.31</v>
       </c>
-      <c r="C6" s="4" t="n">
+      <c r="D6" s="4" t="n">
         <v>119.49</v>
       </c>
-      <c r="D6" s="5" t="n">
+      <c r="E6" s="5" t="n">
         <v>23052228</v>
       </c>
-      <c r="E6" t="inlineStr"/>
+      <c r="F6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" s="2" t="n">
         <v>46265</v>
       </c>
-      <c r="B7" s="4" t="n">
+      <c r="B7" s="2" t="n">
+        <v>46265</v>
+      </c>
+      <c r="C7" s="4" t="n">
         <v>118.56</v>
       </c>
-      <c r="C7" s="4" t="n">
+      <c r="D7" s="4" t="n">
         <v>116.78</v>
       </c>
-      <c r="D7" s="5" t="n">
+      <c r="E7" s="5" t="n">
         <v>64957381</v>
       </c>
-      <c r="E7" t="inlineStr">
+      <c r="F7" t="inlineStr">
         <is>
           <t>Partial 未完整</t>
         </is>

</xml_diff>

<commit_message>
Add IEF as the 10-year Treasury analysis asset with ^TNX as dropdown option
Final project 115(2) names IEF as the analysis proxy; ^TNX stays selectable
as the risk-free rate reference.

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/sample/PortfolioData_W_20260803_20260831_SAMPLE.xlsx
+++ b/sample/PortfolioData_W_20260803_20260831_SAMPLE.xlsx
@@ -19,7 +19,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="VNQ" sheetId="10" state="visible" r:id="rId10"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="GLD" sheetId="11" state="visible" r:id="rId11"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="DBC" sheetId="12" state="visible" r:id="rId12"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="^TNX" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IEF" sheetId="13" state="visible" r:id="rId13"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="2330.TW" sheetId="14" state="visible" r:id="rId14"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="MMM" sheetId="15" state="visible" r:id="rId15"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="AAPL" sheetId="16" state="visible" r:id="rId16"/>
@@ -863,17 +863,17 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>^TNX</t>
+          <t>IEF</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>CBOE Interest Rate 10 Year T Note</t>
+          <t>iShares 7-10 Year Treasury Bond ETF</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>美國 10 年期公債殖利率 US 10Y Yield</t>
+          <t>美國 10 年期公債 US 10Y Treasury</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
@@ -883,7 +883,7 @@
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>殖利率 % Yield</t>
+          <t>價格 Price</t>
         </is>
       </c>
       <c r="F11" s="2" t="n">
@@ -895,11 +895,7 @@
       <c r="H11" t="n">
         <v>6</v>
       </c>
-      <c r="I11" t="inlineStr">
-        <is>
-          <t>殖利率 %，非價格，不可直接計算報酬 / Yield in %, not a price</t>
-        </is>
-      </c>
+      <c r="I11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -1159,14 +1155,14 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>^TNX 為殖利率（%），不是價格，不可直接計算報酬</t>
+          <t>若選擇 ^TNX（取代 IEF）：^TNX 為殖利率（%），不是價格，不可直接計算報酬</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>^TNX is a yield in %, not a price; do not compute returns from it directly</t>
+          <t>If ^TNX is selected (instead of IEF): it is a yield in %, not a price; do not compute returns from it directly</t>
         </is>
       </c>
     </row>
@@ -1841,12 +1837,12 @@
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>Yield (%) 殖利率</t>
+          <t>Close 收盤價</t>
         </is>
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>Adj Yield (%) 調整後殖利率</t>
+          <t>Adj Close 調整後收盤價</t>
         </is>
       </c>
       <c r="E1" s="1" t="inlineStr">
@@ -1868,13 +1864,13 @@
         <v>46234</v>
       </c>
       <c r="C2" s="4" t="n">
-        <v>4.7</v>
+        <v>93.01000000000001</v>
       </c>
       <c r="D2" s="4" t="n">
-        <v>4.7</v>
+        <v>91.61</v>
       </c>
       <c r="E2" s="5" t="n">
-        <v>0</v>
+        <v>52105079</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -1890,13 +1886,13 @@
         <v>46241</v>
       </c>
       <c r="C3" s="4" t="n">
-        <v>4.689</v>
+        <v>91.83</v>
       </c>
       <c r="D3" s="4" t="n">
-        <v>4.689</v>
+        <v>90.45</v>
       </c>
       <c r="E3" s="5" t="n">
-        <v>0</v>
+        <v>26983952</v>
       </c>
       <c r="F3" t="inlineStr"/>
     </row>
@@ -1908,13 +1904,13 @@
         <v>46248</v>
       </c>
       <c r="C4" s="4" t="n">
-        <v>4.647</v>
+        <v>94.25</v>
       </c>
       <c r="D4" s="4" t="n">
-        <v>4.647</v>
+        <v>92.84</v>
       </c>
       <c r="E4" s="5" t="n">
-        <v>0</v>
+        <v>2863698</v>
       </c>
       <c r="F4" t="inlineStr"/>
     </row>
@@ -1926,13 +1922,13 @@
         <v>46255</v>
       </c>
       <c r="C5" s="4" t="n">
-        <v>4.699</v>
+        <v>93.5</v>
       </c>
       <c r="D5" s="4" t="n">
-        <v>4.699</v>
+        <v>92.09999999999999</v>
       </c>
       <c r="E5" s="5" t="n">
-        <v>0</v>
+        <v>64239650</v>
       </c>
       <c r="F5" t="inlineStr"/>
     </row>
@@ -1944,13 +1940,13 @@
         <v>46262</v>
       </c>
       <c r="C6" s="4" t="n">
-        <v>4.64</v>
+        <v>96.15000000000001</v>
       </c>
       <c r="D6" s="4" t="n">
-        <v>4.64</v>
+        <v>94.70999999999999</v>
       </c>
       <c r="E6" s="5" t="n">
-        <v>0</v>
+        <v>12846758</v>
       </c>
       <c r="F6" t="inlineStr"/>
     </row>
@@ -1962,13 +1958,13 @@
         <v>46265</v>
       </c>
       <c r="C7" s="4" t="n">
-        <v>4.646</v>
+        <v>95.34999999999999</v>
       </c>
       <c r="D7" s="4" t="n">
-        <v>4.646</v>
+        <v>93.92</v>
       </c>
       <c r="E7" s="5" t="n">
-        <v>0</v>
+        <v>84765367</v>
       </c>
       <c r="F7" t="inlineStr">
         <is>
@@ -2912,7 +2908,7 @@
       </c>
       <c r="K1" s="1" t="inlineStr">
         <is>
-          <t>^TNX</t>
+          <t>IEF</t>
         </is>
       </c>
       <c r="L1" s="1" t="inlineStr">
@@ -2978,7 +2974,7 @@
         <v>23.28</v>
       </c>
       <c r="K2" s="4" t="n">
-        <v>4.7</v>
+        <v>91.61</v>
       </c>
       <c r="L2" s="4" t="n">
         <v>2380.88</v>
@@ -3033,7 +3029,7 @@
         <v>22.77</v>
       </c>
       <c r="K3" s="4" t="n">
-        <v>4.689</v>
+        <v>90.45</v>
       </c>
       <c r="L3" s="4" t="n">
         <v>2384.13</v>
@@ -3082,7 +3078,7 @@
         <v>22.21</v>
       </c>
       <c r="K4" s="4" t="n">
-        <v>4.647</v>
+        <v>92.84</v>
       </c>
       <c r="L4" s="4" t="n">
         <v>2344.55</v>
@@ -3133,7 +3129,7 @@
         <v>22.72</v>
       </c>
       <c r="K5" s="4" t="n">
-        <v>4.699</v>
+        <v>92.09999999999999</v>
       </c>
       <c r="L5" s="4" t="n">
         <v>2399.73</v>
@@ -3184,7 +3180,7 @@
         <v>22.35</v>
       </c>
       <c r="K6" s="4" t="n">
-        <v>4.64</v>
+        <v>94.70999999999999</v>
       </c>
       <c r="L6" s="4" t="n">
         <v>2454.18</v>
@@ -3235,7 +3231,7 @@
         <v>21.72</v>
       </c>
       <c r="K7" s="4" t="n">
-        <v>4.646</v>
+        <v>93.92</v>
       </c>
       <c r="L7" s="4" t="n">
         <v>2463.6</v>
@@ -3344,7 +3340,7 @@
       </c>
       <c r="K1" s="1" t="inlineStr">
         <is>
-          <t>^TNX</t>
+          <t>IEF</t>
         </is>
       </c>
       <c r="L1" s="1" t="inlineStr">
@@ -3410,7 +3406,7 @@
         <v>23.63</v>
       </c>
       <c r="K2" s="4" t="n">
-        <v>4.7</v>
+        <v>93.01000000000001</v>
       </c>
       <c r="L2" s="4" t="n">
         <v>2417.14</v>
@@ -3465,7 +3461,7 @@
         <v>23.12</v>
       </c>
       <c r="K3" s="4" t="n">
-        <v>4.689</v>
+        <v>91.83</v>
       </c>
       <c r="L3" s="4" t="n">
         <v>2420.44</v>
@@ -3514,7 +3510,7 @@
         <v>22.55</v>
       </c>
       <c r="K4" s="4" t="n">
-        <v>4.647</v>
+        <v>94.25</v>
       </c>
       <c r="L4" s="4" t="n">
         <v>2380.25</v>
@@ -3565,7 +3561,7 @@
         <v>23.07</v>
       </c>
       <c r="K5" s="4" t="n">
-        <v>4.699</v>
+        <v>93.5</v>
       </c>
       <c r="L5" s="4" t="n">
         <v>2436.27</v>
@@ -3616,7 +3612,7 @@
         <v>22.69</v>
       </c>
       <c r="K6" s="4" t="n">
-        <v>4.64</v>
+        <v>96.15000000000001</v>
       </c>
       <c r="L6" s="4" t="n">
         <v>2491.55</v>
@@ -3667,7 +3663,7 @@
         <v>22.05</v>
       </c>
       <c r="K7" s="4" t="n">
-        <v>4.646</v>
+        <v>95.34999999999999</v>
       </c>
       <c r="L7" s="4" t="n">
         <v>2501.12</v>

</xml_diff>

<commit_message>
Make ^TNX an independent opt-in checkbox next to IEF
IEF is the 10-year Treasury analysis asset; ^TNX is the risk-free rate
reference, unchecked by default and excluded from the 15-asset matrix.

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/sample/PortfolioData_W_20260803_20260831_SAMPLE.xlsx
+++ b/sample/PortfolioData_W_20260803_20260831_SAMPLE.xlsx
@@ -20,11 +20,12 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="GLD" sheetId="11" state="visible" r:id="rId11"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="DBC" sheetId="12" state="visible" r:id="rId12"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IEF" sheetId="13" state="visible" r:id="rId13"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="2330.TW" sheetId="14" state="visible" r:id="rId14"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="MMM" sheetId="15" state="visible" r:id="rId15"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="AAPL" sheetId="16" state="visible" r:id="rId16"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="JPM" sheetId="17" state="visible" r:id="rId17"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="LVMUY" sheetId="18" state="visible" r:id="rId18"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="^TNX" sheetId="14" state="visible" r:id="rId14"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="2330.TW" sheetId="15" state="visible" r:id="rId15"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="MMM" sheetId="16" state="visible" r:id="rId16"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="AAPL" sheetId="17" state="visible" r:id="rId17"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="JPM" sheetId="18" state="visible" r:id="rId18"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="LVMUY" sheetId="19" state="visible" r:id="rId19"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -458,7 +459,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I47"/>
+  <dimension ref="A1:I48"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -900,27 +901,27 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>2330.TW</t>
+          <t>^TNX</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Taiwan Semiconductor Manufacturing</t>
+          <t>CBOE Interest Rate 10 Year T Note</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>個股 Stock</t>
+          <t>美國 10 年期公債殖利率（無風險利率，不計入 15 檔）US 10Y Yield (risk-free, not in the 15)</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>TWD</t>
+          <t>USD</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>價格 Price</t>
+          <t>殖利率 % Yield</t>
         </is>
       </c>
       <c r="F12" s="2" t="n">
@@ -932,17 +933,21 @@
       <c r="H12" t="n">
         <v>6</v>
       </c>
-      <c r="I12" t="inlineStr"/>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>殖利率 %，非價格；無風險利率參考，算 15×15 矩陣時請排除 / Yield in %, not a price; risk-free reference, exclude from the 15x15 matrix</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>MMM</t>
+          <t>2330.TW</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>3M Company</t>
+          <t>Taiwan Semiconductor Manufacturing</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -952,7 +957,7 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>USD</t>
+          <t>TWD</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
@@ -974,12 +979,12 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>AAPL</t>
+          <t>MMM</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Apple Inc.</t>
+          <t>3M Company</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -1011,12 +1016,12 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>JPM</t>
+          <t>AAPL</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>JPMorgan Chase &amp; Co.</t>
+          <t>Apple Inc.</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -1048,12 +1053,12 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>LVMUY</t>
+          <t>JPM</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>LVMH Moet Hennessy Louis Vuitton (ADR)</t>
+          <t>JPMorgan Chase &amp; Co.</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -1082,211 +1087,248 @@
       </c>
       <c r="I16" t="inlineStr"/>
     </row>
-    <row r="18">
-      <c r="A18" s="3" t="inlineStr">
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>LVMUY</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>LVMH Moet Hennessy Louis Vuitton (ADR)</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>個股 Stock</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>價格 Price</t>
+        </is>
+      </c>
+      <c r="F17" s="2" t="n">
+        <v>46234</v>
+      </c>
+      <c r="G17" s="2" t="n">
+        <v>46265</v>
+      </c>
+      <c r="H17" t="n">
+        <v>6</v>
+      </c>
+      <c r="I17" t="inlineStr"/>
+    </row>
+    <row r="19">
+      <c r="A19" s="3" t="inlineStr">
         <is>
           <t>【這是範例檔 SAMPLE】數字是隨機產生的假資料，只用來確認版面，不可用於報告。</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" t="inlineStr">
-        <is>
-          <t>THIS IS A SAMPLE FILE. Numbers are random dummy data, for layout review only.</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>資料來源：Yahoo Finance；下載時間：2026-10-08 12:00（台北時間）</t>
+          <t>THIS IS A SAMPLE FILE. Numbers are random dummy data, for layout review only.</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Source: Yahoo Finance; downloaded at 2026-10-08 12:00 (Taipei time)</t>
+          <t>資料來源：Yahoo Finance；下載時間：2026-10-08 12:00（台北時間）</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>頻率：週 Weekly；期間：2026-08-03 ~ 2026-08-31（往回推：一個月）</t>
+          <t>Source: Yahoo Finance; downloaded at 2026-10-08 12:00 (Taipei time)</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Frequency: Weekly; period: 2026-08-03 ~ 2026-08-31 (lookback: one month)</t>
+          <t>頻率：週 Weekly；期間：2026-08-03 ~ 2026-08-31（往回推：一個月）</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Close = 未調整股利（已調整分割）；Adj Close = 調整分割與股利</t>
+          <t>Frequency: Weekly; period: 2026-08-03 ~ 2026-08-31 (lookback: one month)</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Close = not adjusted for dividends (split-adjusted); Adj Close = adjusted for splits and dividends</t>
+          <t>Close = 未調整股利（已調整分割）；Adj Close = 調整分割與股利</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>幣別：各標的維持當地幣別，未換匯</t>
+          <t>Close = not adjusted for dividends (split-adjusted); Adj Close = adjusted for splits and dividends</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Currency: each series stays in its local currency; no FX conversion</t>
+          <t>幣別：各標的維持當地幣別，未換匯</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>若選擇 ^TNX（取代 IEF）：^TNX 為殖利率（%），不是價格，不可直接計算報酬</t>
+          <t>Currency: each series stays in its local currency; no FX conversion</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>If ^TNX is selected (instead of IEF): it is a yield in %, not a price; do not compute returns from it directly</t>
+          <t>^TNX（若有勾選）為殖利率（%），不是價格，不可直接計算報酬，也不計入 15 檔共變異數矩陣</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>兩個日期欄：Period 期間 = 對齊日（日資料為當天、週資料為該週週一、月資料為該月 1 日、年資料為 1/1，與雅虎財經的日期標示相同），所有標的分頁與 Combined 分頁都一樣；Trade Date 取值日 = 收盤價實際來自哪一天（該期最後一個交易日；結束日落在期中時，為截至結束日最新的一天）</t>
+          <t>^TNX (if selected) is a yield in %, not a price; do not compute returns from it directly, and exclude it from the 15x15 covariance matrix</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>Two date columns: Period = alignment date (that week's Monday, the 1st of the month, Jan 1, or the day itself for daily data), identical in every sheet; Trade Date = the day Close/Adj Close actually come from (the last trading day of the period)</t>
+          <t>兩個日期欄：Period 期間 = 對齊日（日資料為當天、週資料為該週週一、月資料為該月 1 日、年資料為 1/1，與雅虎財經的日期標示相同），所有標的分頁與 Combined 分頁都一樣；Trade Date 取值日 = 收盤價實際來自哪一天（該期最後一個交易日；結束日落在期中時，為截至結束日最新的一天）</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>收盤價與調整後收盤價取該期最後一個交易日的值，成交量為整期加總</t>
+          <t>Two date columns: Period = alignment date (that week's Monday, the 1st of the month, Jan 1, or the day itself for daily data), identical in every sheet; Trade Date = the day Close/Adj Close actually come from (the last trading day of the period)</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>Close and Adj Close are from the last trading day of the period; Volume is the total over the period</t>
+          <t>收盤價與調整後收盤價取該期最後一個交易日的值，成交量為整期加總</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>Combined 對齊：日資料以交易日；週資料以該週週一；月資料以月初；年資料以 1/1</t>
+          <t>Close and Adj Close are from the last trading day of the period; Volume is the total over the period</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>Combined alignment: daily = trading day; weekly = that week's Monday; monthly = first of the month; yearly = Jan 1</t>
+          <t>Combined 對齊：日資料以交易日；週資料以該週週一；月資料以月初；年資料以 1/1</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>所有分頁的列相同：列 = 所有已下載標的的期間聯集。某標的該期沒有交易時，該列只填 Period，取值日與數值留白，Flag 標 No trading 休市；標的尚未有資料的期間標 No data 無資料。所有標的都沒有交易的期間不會出現</t>
+          <t>Combined alignment: daily = trading day; weekly = that week's Monday; monthly = first of the month; yearly = Jan 1</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>All sheets share the same rows (union of periods). When a ticker has no trading in a period, only Period is filled, Trade Date and values are blank, and Flag says No trading; earlier periods are flagged No data</t>
+          <t>所有分頁的列相同：列 = 所有已下載標的的期間聯集。某標的該期沒有交易時，該列只填 Period，取值日與數值留白，Flag 標 No trading 休市；標的尚未有資料的期間標 No data 無資料。所有標的都沒有交易的期間不會出現</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>空白格不補值。以公式計算報酬或共變異數前，請自行處理（例如以 Flag 篩選掉空白列）</t>
+          <t>All sheets share the same rows (union of periods). When a ticker has no trading in a period, only Period is filled, Trade Date and values are blank, and Flag says No trading; earlier periods are flagged No data</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>Blank cells are not filled. Handle them yourself (e.g. filter out blank rows using Flag) before computing returns or covariances</t>
+          <t>空白格不補值。以公式計算報酬或共變異數前，請自行處理（例如以 Flag 篩選掉空白列）</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>Flag 註記：No trading 休市 = 該標的在該期沒有交易；No data 無資料 = 該標的在該期之前尚無資料</t>
+          <t>Blank cells are not filled. Handle them yourself (e.g. filter out blank rows using Flag) before computing returns or covariances</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>Flag: No trading = the ticker has no trading in that period; No data = no data before this period</t>
+          <t>Flag 註記：No trading 休市 = 該標的在該期沒有交易；No data 無資料 = 該標的在該期之前尚無資料</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>Flag 註記：Prior period 前一期 = 起始日之前多抓的一期，供計算第一期報酬</t>
+          <t>Flag: No trading = the ticker has no trading in that period; No data = no data before this period</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>Flag: Prior period = one extra period before the start date, for computing the first return</t>
+          <t>Flag 註記：Prior period 前一期 = 起始日之前多抓的一期，供計算第一期報酬</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>Flag 註記：Partial 未完整 = 結束日落在週期中間，該期資料不完整（收盤價取截至結束日最新的一天）</t>
+          <t>Flag: Prior period = one extra period before the start date, for computing the first return</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>Flag: Partial = the end date falls inside the period; the period is incomplete (values are from the latest trading day up to the end date)</t>
+          <t>Flag 註記：Partial 未完整 = 結束日落在週期中間，該期資料不完整（收盤價取截至結束日最新的一天）</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>Flag 註記：Intraday 盤中 = 日資料最後一筆為當日尚未收盤的盤中價</t>
+          <t>Flag: Partial = the end date falls inside the period; the period is incomplete (values are from the latest trading day up to the end date)</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
+        <is>
+          <t>Flag 註記：Intraday 盤中 = 日資料最後一筆為當日尚未收盤的盤中價</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
         <is>
           <t>Flag: Intraday = the last daily row is an unfinished intraday price</t>
         </is>
@@ -2007,12 +2049,12 @@
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>Close 收盤價</t>
+          <t>Yield (%) 殖利率</t>
         </is>
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>Adj Close 調整後收盤價</t>
+          <t>Adj Yield (%) 調整後殖利率</t>
         </is>
       </c>
       <c r="E1" s="1" t="inlineStr">
@@ -2034,13 +2076,13 @@
         <v>46234</v>
       </c>
       <c r="C2" s="4" t="n">
-        <v>2417.14</v>
+        <v>4.714</v>
       </c>
       <c r="D2" s="4" t="n">
-        <v>2380.88</v>
+        <v>4.714</v>
       </c>
       <c r="E2" s="5" t="n">
-        <v>59564514</v>
+        <v>0</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -2056,13 +2098,13 @@
         <v>46241</v>
       </c>
       <c r="C3" s="4" t="n">
-        <v>2420.44</v>
+        <v>4.71</v>
       </c>
       <c r="D3" s="4" t="n">
-        <v>2384.13</v>
+        <v>4.71</v>
       </c>
       <c r="E3" s="5" t="n">
-        <v>3990777</v>
+        <v>0</v>
       </c>
       <c r="F3" t="inlineStr"/>
     </row>
@@ -2074,13 +2116,13 @@
         <v>46248</v>
       </c>
       <c r="C4" s="4" t="n">
-        <v>2380.25</v>
+        <v>4.725</v>
       </c>
       <c r="D4" s="4" t="n">
-        <v>2344.55</v>
+        <v>4.725</v>
       </c>
       <c r="E4" s="5" t="n">
-        <v>67940689</v>
+        <v>0</v>
       </c>
       <c r="F4" t="inlineStr"/>
     </row>
@@ -2092,13 +2134,13 @@
         <v>46255</v>
       </c>
       <c r="C5" s="4" t="n">
-        <v>2436.27</v>
+        <v>4.692</v>
       </c>
       <c r="D5" s="4" t="n">
-        <v>2399.73</v>
+        <v>4.692</v>
       </c>
       <c r="E5" s="5" t="n">
-        <v>89707598</v>
+        <v>0</v>
       </c>
       <c r="F5" t="inlineStr"/>
     </row>
@@ -2110,13 +2152,13 @@
         <v>46262</v>
       </c>
       <c r="C6" s="4" t="n">
-        <v>2491.55</v>
+        <v>4.738</v>
       </c>
       <c r="D6" s="4" t="n">
-        <v>2454.18</v>
+        <v>4.738</v>
       </c>
       <c r="E6" s="5" t="n">
-        <v>6617569</v>
+        <v>0</v>
       </c>
       <c r="F6" t="inlineStr"/>
     </row>
@@ -2128,13 +2170,13 @@
         <v>46265</v>
       </c>
       <c r="C7" s="4" t="n">
-        <v>2501.12</v>
+        <v>4.785</v>
       </c>
       <c r="D7" s="4" t="n">
-        <v>2463.6</v>
+        <v>4.785</v>
       </c>
       <c r="E7" s="5" t="n">
-        <v>45992922</v>
+        <v>0</v>
       </c>
       <c r="F7" t="inlineStr">
         <is>
@@ -2204,10 +2246,10 @@
         <v>46234</v>
       </c>
       <c r="C2" s="4" t="n">
-        <v>149.91</v>
+        <v>2398.57</v>
       </c>
       <c r="D2" s="4" t="n">
-        <v>147.66</v>
+        <v>2362.59</v>
       </c>
       <c r="E2" s="5" t="n">
         <v>77131377</v>
@@ -2226,10 +2268,10 @@
         <v>46241</v>
       </c>
       <c r="C3" s="4" t="n">
-        <v>153.76</v>
+        <v>2460.21</v>
       </c>
       <c r="D3" s="4" t="n">
-        <v>151.45</v>
+        <v>2423.31</v>
       </c>
       <c r="E3" s="5" t="n">
         <v>64498494</v>
@@ -2244,10 +2286,10 @@
         <v>46248</v>
       </c>
       <c r="C4" s="4" t="n">
-        <v>153.67</v>
+        <v>2458.65</v>
       </c>
       <c r="D4" s="4" t="n">
-        <v>151.36</v>
+        <v>2421.77</v>
       </c>
       <c r="E4" s="5" t="n">
         <v>80837457</v>
@@ -2262,10 +2304,10 @@
         <v>46255</v>
       </c>
       <c r="C5" s="4" t="n">
-        <v>150.95</v>
+        <v>2415.24</v>
       </c>
       <c r="D5" s="4" t="n">
-        <v>148.69</v>
+        <v>2379.01</v>
       </c>
       <c r="E5" s="5" t="n">
         <v>70707214</v>
@@ -2280,10 +2322,10 @@
         <v>46262</v>
       </c>
       <c r="C6" s="4" t="n">
-        <v>151.09</v>
+        <v>2417.48</v>
       </c>
       <c r="D6" s="4" t="n">
-        <v>148.82</v>
+        <v>2381.22</v>
       </c>
       <c r="E6" s="5" t="n">
         <v>84404159</v>
@@ -2298,10 +2340,10 @@
         <v>46265</v>
       </c>
       <c r="C7" s="4" t="n">
-        <v>154.35</v>
+        <v>2469.56</v>
       </c>
       <c r="D7" s="4" t="n">
-        <v>152.03</v>
+        <v>2432.52</v>
       </c>
       <c r="E7" s="5" t="n">
         <v>14633036</v>
@@ -2374,10 +2416,10 @@
         <v>46234</v>
       </c>
       <c r="C2" s="4" t="n">
-        <v>230.19</v>
+        <v>150.13</v>
       </c>
       <c r="D2" s="4" t="n">
-        <v>226.74</v>
+        <v>147.88</v>
       </c>
       <c r="E2" s="5" t="n">
         <v>73018730</v>
@@ -2396,10 +2438,10 @@
         <v>46241</v>
       </c>
       <c r="C3" s="4" t="n">
-        <v>233.26</v>
+        <v>152.13</v>
       </c>
       <c r="D3" s="4" t="n">
-        <v>229.76</v>
+        <v>149.85</v>
       </c>
       <c r="E3" s="5" t="n">
         <v>21139495</v>
@@ -2414,10 +2456,10 @@
         <v>46248</v>
       </c>
       <c r="C4" s="4" t="n">
-        <v>232.05</v>
+        <v>151.34</v>
       </c>
       <c r="D4" s="4" t="n">
-        <v>228.57</v>
+        <v>149.07</v>
       </c>
       <c r="E4" s="5" t="n">
         <v>52298696</v>
@@ -2432,10 +2474,10 @@
         <v>46255</v>
       </c>
       <c r="C5" s="4" t="n">
-        <v>232.37</v>
+        <v>151.54</v>
       </c>
       <c r="D5" s="4" t="n">
-        <v>228.88</v>
+        <v>149.27</v>
       </c>
       <c r="E5" s="5" t="n">
         <v>88356860</v>
@@ -2450,10 +2492,10 @@
         <v>46262</v>
       </c>
       <c r="C6" s="4" t="n">
-        <v>237.63</v>
+        <v>154.98</v>
       </c>
       <c r="D6" s="4" t="n">
-        <v>234.07</v>
+        <v>152.66</v>
       </c>
       <c r="E6" s="5" t="n">
         <v>82726197</v>
@@ -2468,10 +2510,10 @@
         <v>46265</v>
       </c>
       <c r="C7" s="4" t="n">
-        <v>234.02</v>
+        <v>152.62</v>
       </c>
       <c r="D7" s="4" t="n">
-        <v>230.51</v>
+        <v>150.33</v>
       </c>
       <c r="E7" s="5" t="n">
         <v>2223590</v>
@@ -2544,10 +2586,10 @@
         <v>46234</v>
       </c>
       <c r="C2" s="4" t="n">
-        <v>286.18</v>
+        <v>226.97</v>
       </c>
       <c r="D2" s="4" t="n">
-        <v>281.89</v>
+        <v>223.57</v>
       </c>
       <c r="E2" s="5" t="n">
         <v>26927476</v>
@@ -2566,10 +2608,10 @@
         <v>46241</v>
       </c>
       <c r="C3" s="4" t="n">
-        <v>289.73</v>
+        <v>229.78</v>
       </c>
       <c r="D3" s="4" t="n">
-        <v>285.38</v>
+        <v>226.33</v>
       </c>
       <c r="E3" s="5" t="n">
         <v>21751469</v>
@@ -2584,10 +2626,10 @@
         <v>46248</v>
       </c>
       <c r="C4" s="4" t="n">
-        <v>297.4</v>
+        <v>235.87</v>
       </c>
       <c r="D4" s="4" t="n">
-        <v>292.94</v>
+        <v>232.33</v>
       </c>
       <c r="E4" s="5" t="n">
         <v>88027814</v>
@@ -2602,10 +2644,10 @@
         <v>46255</v>
       </c>
       <c r="C5" s="4" t="n">
-        <v>302.67</v>
+        <v>240.05</v>
       </c>
       <c r="D5" s="4" t="n">
-        <v>298.13</v>
+        <v>236.45</v>
       </c>
       <c r="E5" s="5" t="n">
         <v>19476896</v>
@@ -2620,10 +2662,10 @@
         <v>46262</v>
       </c>
       <c r="C6" s="4" t="n">
-        <v>294.98</v>
+        <v>233.95</v>
       </c>
       <c r="D6" s="4" t="n">
-        <v>290.56</v>
+        <v>230.44</v>
       </c>
       <c r="E6" s="5" t="n">
         <v>30710182</v>
@@ -2638,10 +2680,10 @@
         <v>46265</v>
       </c>
       <c r="C7" s="4" t="n">
-        <v>300.41</v>
+        <v>238.26</v>
       </c>
       <c r="D7" s="4" t="n">
-        <v>295.9</v>
+        <v>234.69</v>
       </c>
       <c r="E7" s="5" t="n">
         <v>6023039</v>
@@ -2714,10 +2756,10 @@
         <v>46234</v>
       </c>
       <c r="C2" s="4" t="n">
-        <v>117.23</v>
+        <v>283.31</v>
       </c>
       <c r="D2" s="4" t="n">
-        <v>115.47</v>
+        <v>279.06</v>
       </c>
       <c r="E2" s="5" t="n">
         <v>89515598</v>
@@ -2736,10 +2778,10 @@
         <v>46241</v>
       </c>
       <c r="C3" s="4" t="n">
-        <v>117.73</v>
+        <v>284.52</v>
       </c>
       <c r="D3" s="4" t="n">
-        <v>115.96</v>
+        <v>280.25</v>
       </c>
       <c r="E3" s="5" t="n">
         <v>35143088</v>
@@ -2754,10 +2796,10 @@
         <v>46248</v>
       </c>
       <c r="C4" s="4" t="n">
-        <v>116.28</v>
+        <v>281</v>
       </c>
       <c r="D4" s="4" t="n">
-        <v>114.54</v>
+        <v>276.78</v>
       </c>
       <c r="E4" s="5" t="n">
         <v>36329608</v>
@@ -2772,10 +2814,10 @@
         <v>46255</v>
       </c>
       <c r="C5" s="4" t="n">
-        <v>114.99</v>
+        <v>277.89</v>
       </c>
       <c r="D5" s="4" t="n">
-        <v>113.27</v>
+        <v>273.72</v>
       </c>
       <c r="E5" s="5" t="n">
         <v>11747679</v>
@@ -2790,10 +2832,10 @@
         <v>46262</v>
       </c>
       <c r="C6" s="4" t="n">
-        <v>116.46</v>
+        <v>281.44</v>
       </c>
       <c r="D6" s="4" t="n">
-        <v>114.71</v>
+        <v>277.22</v>
       </c>
       <c r="E6" s="5" t="n">
         <v>42666357</v>
@@ -2808,13 +2850,183 @@
         <v>46265</v>
       </c>
       <c r="C7" s="4" t="n">
-        <v>116.5</v>
+        <v>281.53</v>
       </c>
       <c r="D7" s="4" t="n">
-        <v>114.75</v>
+        <v>277.31</v>
       </c>
       <c r="E7" s="5" t="n">
         <v>55240635</v>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>Partial 未完整</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F7"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="13" customWidth="1" min="1" max="1"/>
+    <col width="15" customWidth="1" min="2" max="2"/>
+    <col width="16" customWidth="1" min="3" max="3"/>
+    <col width="24" customWidth="1" min="4" max="4"/>
+    <col width="16" customWidth="1" min="5" max="5"/>
+    <col width="22" customWidth="1" min="6" max="6"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="32" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Period 期間</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Trade Date 取值日</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Close 收盤價</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Adj Close 調整後收盤價</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Volume 成交量</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Flag 註記</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="n">
+        <v>46230</v>
+      </c>
+      <c r="B2" s="2" t="n">
+        <v>46234</v>
+      </c>
+      <c r="C2" s="4" t="n">
+        <v>123.93</v>
+      </c>
+      <c r="D2" s="4" t="n">
+        <v>122.07</v>
+      </c>
+      <c r="E2" s="5" t="n">
+        <v>3564266</v>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>Prior period 前一期</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="n">
+        <v>46237</v>
+      </c>
+      <c r="B3" s="2" t="n">
+        <v>46241</v>
+      </c>
+      <c r="C3" s="4" t="n">
+        <v>124.41</v>
+      </c>
+      <c r="D3" s="4" t="n">
+        <v>122.54</v>
+      </c>
+      <c r="E3" s="5" t="n">
+        <v>6855520</v>
+      </c>
+      <c r="F3" t="inlineStr"/>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="n">
+        <v>46244</v>
+      </c>
+      <c r="B4" s="2" t="n">
+        <v>46248</v>
+      </c>
+      <c r="C4" s="4" t="n">
+        <v>121.96</v>
+      </c>
+      <c r="D4" s="4" t="n">
+        <v>120.13</v>
+      </c>
+      <c r="E4" s="5" t="n">
+        <v>34071323</v>
+      </c>
+      <c r="F4" t="inlineStr"/>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="n">
+        <v>46251</v>
+      </c>
+      <c r="B5" s="2" t="n">
+        <v>46255</v>
+      </c>
+      <c r="C5" s="4" t="n">
+        <v>118.43</v>
+      </c>
+      <c r="D5" s="4" t="n">
+        <v>116.65</v>
+      </c>
+      <c r="E5" s="5" t="n">
+        <v>21763339</v>
+      </c>
+      <c r="F5" t="inlineStr"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="n">
+        <v>46258</v>
+      </c>
+      <c r="B6" s="2" t="n">
+        <v>46262</v>
+      </c>
+      <c r="C6" s="4" t="n">
+        <v>121.48</v>
+      </c>
+      <c r="D6" s="4" t="n">
+        <v>119.66</v>
+      </c>
+      <c r="E6" s="5" t="n">
+        <v>51297169</v>
+      </c>
+      <c r="F6" t="inlineStr"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="n">
+        <v>46265</v>
+      </c>
+      <c r="B7" s="2" t="n">
+        <v>46265</v>
+      </c>
+      <c r="C7" s="4" t="n">
+        <v>119.73</v>
+      </c>
+      <c r="D7" s="4" t="n">
+        <v>117.93</v>
+      </c>
+      <c r="E7" s="5" t="n">
+        <v>47376028</v>
       </c>
       <c r="F7" t="inlineStr">
         <is>
@@ -2833,7 +3045,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q7"/>
+  <dimension ref="A1:R7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -2852,7 +3064,8 @@
     <col width="11" customWidth="1" min="14" max="14"/>
     <col width="11" customWidth="1" min="15" max="15"/>
     <col width="11" customWidth="1" min="16" max="16"/>
-    <col width="20" customWidth="1" min="17" max="17"/>
+    <col width="11" customWidth="1" min="17" max="17"/>
+    <col width="20" customWidth="1" min="18" max="18"/>
   </cols>
   <sheetData>
     <row r="1" ht="32" customHeight="1">
@@ -2913,30 +3126,35 @@
       </c>
       <c r="L1" s="1" t="inlineStr">
         <is>
+          <t>^TNX</t>
+        </is>
+      </c>
+      <c r="M1" s="1" t="inlineStr">
+        <is>
           <t>2330.TW</t>
         </is>
       </c>
-      <c r="M1" s="1" t="inlineStr">
+      <c r="N1" s="1" t="inlineStr">
         <is>
           <t>MMM</t>
         </is>
       </c>
-      <c r="N1" s="1" t="inlineStr">
+      <c r="O1" s="1" t="inlineStr">
         <is>
           <t>AAPL</t>
         </is>
       </c>
-      <c r="O1" s="1" t="inlineStr">
+      <c r="P1" s="1" t="inlineStr">
         <is>
           <t>JPM</t>
         </is>
       </c>
-      <c r="P1" s="1" t="inlineStr">
+      <c r="Q1" s="1" t="inlineStr">
         <is>
           <t>LVMUY</t>
         </is>
       </c>
-      <c r="Q1" s="1" t="inlineStr">
+      <c r="R1" s="1" t="inlineStr">
         <is>
           <t>Flag 註記</t>
         </is>
@@ -2977,21 +3195,24 @@
         <v>91.61</v>
       </c>
       <c r="L2" s="4" t="n">
-        <v>2380.88</v>
+        <v>4.714</v>
       </c>
       <c r="M2" s="4" t="n">
-        <v>147.66</v>
+        <v>2362.59</v>
       </c>
       <c r="N2" s="4" t="n">
-        <v>226.74</v>
+        <v>147.88</v>
       </c>
       <c r="O2" s="4" t="n">
-        <v>281.89</v>
+        <v>223.57</v>
       </c>
       <c r="P2" s="4" t="n">
-        <v>115.47</v>
-      </c>
-      <c r="Q2" t="inlineStr">
+        <v>279.06</v>
+      </c>
+      <c r="Q2" s="4" t="n">
+        <v>122.07</v>
+      </c>
+      <c r="R2" t="inlineStr">
         <is>
           <t>Prior period 前一期</t>
         </is>
@@ -3032,21 +3253,24 @@
         <v>90.45</v>
       </c>
       <c r="L3" s="4" t="n">
-        <v>2384.13</v>
+        <v>4.71</v>
       </c>
       <c r="M3" s="4" t="n">
-        <v>151.45</v>
+        <v>2423.31</v>
       </c>
       <c r="N3" s="4" t="n">
-        <v>229.76</v>
+        <v>149.85</v>
       </c>
       <c r="O3" s="4" t="n">
-        <v>285.38</v>
+        <v>226.33</v>
       </c>
       <c r="P3" s="4" t="n">
-        <v>115.96</v>
-      </c>
-      <c r="Q3" t="inlineStr"/>
+        <v>280.25</v>
+      </c>
+      <c r="Q3" s="4" t="n">
+        <v>122.54</v>
+      </c>
+      <c r="R3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" s="2" t="n">
@@ -3081,21 +3305,24 @@
         <v>92.84</v>
       </c>
       <c r="L4" s="4" t="n">
-        <v>2344.55</v>
+        <v>4.725</v>
       </c>
       <c r="M4" s="4" t="n">
-        <v>151.36</v>
+        <v>2421.77</v>
       </c>
       <c r="N4" s="4" t="n">
-        <v>228.57</v>
+        <v>149.07</v>
       </c>
       <c r="O4" s="4" t="n">
-        <v>292.94</v>
+        <v>232.33</v>
       </c>
       <c r="P4" s="4" t="n">
-        <v>114.54</v>
-      </c>
-      <c r="Q4" t="inlineStr"/>
+        <v>276.78</v>
+      </c>
+      <c r="Q4" s="4" t="n">
+        <v>120.13</v>
+      </c>
+      <c r="R4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" s="2" t="n">
@@ -3132,21 +3359,24 @@
         <v>92.09999999999999</v>
       </c>
       <c r="L5" s="4" t="n">
-        <v>2399.73</v>
+        <v>4.692</v>
       </c>
       <c r="M5" s="4" t="n">
-        <v>148.69</v>
+        <v>2379.01</v>
       </c>
       <c r="N5" s="4" t="n">
-        <v>228.88</v>
+        <v>149.27</v>
       </c>
       <c r="O5" s="4" t="n">
-        <v>298.13</v>
+        <v>236.45</v>
       </c>
       <c r="P5" s="4" t="n">
-        <v>113.27</v>
-      </c>
-      <c r="Q5" t="inlineStr"/>
+        <v>273.72</v>
+      </c>
+      <c r="Q5" s="4" t="n">
+        <v>116.65</v>
+      </c>
+      <c r="R5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" s="2" t="n">
@@ -3183,21 +3413,24 @@
         <v>94.70999999999999</v>
       </c>
       <c r="L6" s="4" t="n">
-        <v>2454.18</v>
+        <v>4.738</v>
       </c>
       <c r="M6" s="4" t="n">
-        <v>148.82</v>
+        <v>2381.22</v>
       </c>
       <c r="N6" s="4" t="n">
-        <v>234.07</v>
+        <v>152.66</v>
       </c>
       <c r="O6" s="4" t="n">
-        <v>290.56</v>
+        <v>230.44</v>
       </c>
       <c r="P6" s="4" t="n">
-        <v>114.71</v>
-      </c>
-      <c r="Q6" t="inlineStr"/>
+        <v>277.22</v>
+      </c>
+      <c r="Q6" s="4" t="n">
+        <v>119.66</v>
+      </c>
+      <c r="R6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" s="2" t="n">
@@ -3234,21 +3467,24 @@
         <v>93.92</v>
       </c>
       <c r="L7" s="4" t="n">
-        <v>2463.6</v>
+        <v>4.785</v>
       </c>
       <c r="M7" s="4" t="n">
-        <v>152.03</v>
+        <v>2432.52</v>
       </c>
       <c r="N7" s="4" t="n">
-        <v>230.51</v>
+        <v>150.33</v>
       </c>
       <c r="O7" s="4" t="n">
-        <v>295.9</v>
+        <v>234.69</v>
       </c>
       <c r="P7" s="4" t="n">
-        <v>114.75</v>
-      </c>
-      <c r="Q7" t="inlineStr">
+        <v>277.31</v>
+      </c>
+      <c r="Q7" s="4" t="n">
+        <v>117.93</v>
+      </c>
+      <c r="R7" t="inlineStr">
         <is>
           <t>Partial 未完整</t>
         </is>
@@ -3265,7 +3501,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q7"/>
+  <dimension ref="A1:R7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -3284,7 +3520,8 @@
     <col width="11" customWidth="1" min="14" max="14"/>
     <col width="11" customWidth="1" min="15" max="15"/>
     <col width="11" customWidth="1" min="16" max="16"/>
-    <col width="20" customWidth="1" min="17" max="17"/>
+    <col width="11" customWidth="1" min="17" max="17"/>
+    <col width="20" customWidth="1" min="18" max="18"/>
   </cols>
   <sheetData>
     <row r="1" ht="32" customHeight="1">
@@ -3345,30 +3582,35 @@
       </c>
       <c r="L1" s="1" t="inlineStr">
         <is>
+          <t>^TNX</t>
+        </is>
+      </c>
+      <c r="M1" s="1" t="inlineStr">
+        <is>
           <t>2330.TW</t>
         </is>
       </c>
-      <c r="M1" s="1" t="inlineStr">
+      <c r="N1" s="1" t="inlineStr">
         <is>
           <t>MMM</t>
         </is>
       </c>
-      <c r="N1" s="1" t="inlineStr">
+      <c r="O1" s="1" t="inlineStr">
         <is>
           <t>AAPL</t>
         </is>
       </c>
-      <c r="O1" s="1" t="inlineStr">
+      <c r="P1" s="1" t="inlineStr">
         <is>
           <t>JPM</t>
         </is>
       </c>
-      <c r="P1" s="1" t="inlineStr">
+      <c r="Q1" s="1" t="inlineStr">
         <is>
           <t>LVMUY</t>
         </is>
       </c>
-      <c r="Q1" s="1" t="inlineStr">
+      <c r="R1" s="1" t="inlineStr">
         <is>
           <t>Flag 註記</t>
         </is>
@@ -3409,21 +3651,24 @@
         <v>93.01000000000001</v>
       </c>
       <c r="L2" s="4" t="n">
-        <v>2417.14</v>
+        <v>4.714</v>
       </c>
       <c r="M2" s="4" t="n">
-        <v>149.91</v>
+        <v>2398.57</v>
       </c>
       <c r="N2" s="4" t="n">
-        <v>230.19</v>
+        <v>150.13</v>
       </c>
       <c r="O2" s="4" t="n">
-        <v>286.18</v>
+        <v>226.97</v>
       </c>
       <c r="P2" s="4" t="n">
-        <v>117.23</v>
-      </c>
-      <c r="Q2" t="inlineStr">
+        <v>283.31</v>
+      </c>
+      <c r="Q2" s="4" t="n">
+        <v>123.93</v>
+      </c>
+      <c r="R2" t="inlineStr">
         <is>
           <t>Prior period 前一期</t>
         </is>
@@ -3464,21 +3709,24 @@
         <v>91.83</v>
       </c>
       <c r="L3" s="4" t="n">
-        <v>2420.44</v>
+        <v>4.71</v>
       </c>
       <c r="M3" s="4" t="n">
-        <v>153.76</v>
+        <v>2460.21</v>
       </c>
       <c r="N3" s="4" t="n">
-        <v>233.26</v>
+        <v>152.13</v>
       </c>
       <c r="O3" s="4" t="n">
-        <v>289.73</v>
+        <v>229.78</v>
       </c>
       <c r="P3" s="4" t="n">
-        <v>117.73</v>
-      </c>
-      <c r="Q3" t="inlineStr"/>
+        <v>284.52</v>
+      </c>
+      <c r="Q3" s="4" t="n">
+        <v>124.41</v>
+      </c>
+      <c r="R3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" s="2" t="n">
@@ -3513,21 +3761,24 @@
         <v>94.25</v>
       </c>
       <c r="L4" s="4" t="n">
-        <v>2380.25</v>
+        <v>4.725</v>
       </c>
       <c r="M4" s="4" t="n">
-        <v>153.67</v>
+        <v>2458.65</v>
       </c>
       <c r="N4" s="4" t="n">
-        <v>232.05</v>
+        <v>151.34</v>
       </c>
       <c r="O4" s="4" t="n">
-        <v>297.4</v>
+        <v>235.87</v>
       </c>
       <c r="P4" s="4" t="n">
-        <v>116.28</v>
-      </c>
-      <c r="Q4" t="inlineStr"/>
+        <v>281</v>
+      </c>
+      <c r="Q4" s="4" t="n">
+        <v>121.96</v>
+      </c>
+      <c r="R4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" s="2" t="n">
@@ -3564,21 +3815,24 @@
         <v>93.5</v>
       </c>
       <c r="L5" s="4" t="n">
-        <v>2436.27</v>
+        <v>4.692</v>
       </c>
       <c r="M5" s="4" t="n">
-        <v>150.95</v>
+        <v>2415.24</v>
       </c>
       <c r="N5" s="4" t="n">
-        <v>232.37</v>
+        <v>151.54</v>
       </c>
       <c r="O5" s="4" t="n">
-        <v>302.67</v>
+        <v>240.05</v>
       </c>
       <c r="P5" s="4" t="n">
-        <v>114.99</v>
-      </c>
-      <c r="Q5" t="inlineStr"/>
+        <v>277.89</v>
+      </c>
+      <c r="Q5" s="4" t="n">
+        <v>118.43</v>
+      </c>
+      <c r="R5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" s="2" t="n">
@@ -3615,21 +3869,24 @@
         <v>96.15000000000001</v>
       </c>
       <c r="L6" s="4" t="n">
-        <v>2491.55</v>
+        <v>4.738</v>
       </c>
       <c r="M6" s="4" t="n">
-        <v>151.09</v>
+        <v>2417.48</v>
       </c>
       <c r="N6" s="4" t="n">
-        <v>237.63</v>
+        <v>154.98</v>
       </c>
       <c r="O6" s="4" t="n">
-        <v>294.98</v>
+        <v>233.95</v>
       </c>
       <c r="P6" s="4" t="n">
-        <v>116.46</v>
-      </c>
-      <c r="Q6" t="inlineStr"/>
+        <v>281.44</v>
+      </c>
+      <c r="Q6" s="4" t="n">
+        <v>121.48</v>
+      </c>
+      <c r="R6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" s="2" t="n">
@@ -3666,21 +3923,24 @@
         <v>95.34999999999999</v>
       </c>
       <c r="L7" s="4" t="n">
-        <v>2501.12</v>
+        <v>4.785</v>
       </c>
       <c r="M7" s="4" t="n">
-        <v>154.35</v>
+        <v>2469.56</v>
       </c>
       <c r="N7" s="4" t="n">
-        <v>234.02</v>
+        <v>152.62</v>
       </c>
       <c r="O7" s="4" t="n">
-        <v>300.41</v>
+        <v>238.26</v>
       </c>
       <c r="P7" s="4" t="n">
-        <v>116.5</v>
-      </c>
-      <c r="Q7" t="inlineStr">
+        <v>281.53</v>
+      </c>
+      <c r="Q7" s="4" t="n">
+        <v>119.73</v>
+      </c>
+      <c r="R7" t="inlineStr">
         <is>
           <t>Partial 未完整</t>
         </is>

</xml_diff>